<commit_message>
Built morning email report generator - still missing intakes and outcomes
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -452,7 +452,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -468,7 +468,7 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -484,7 +484,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -500,7 +500,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>23</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -516,7 +516,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -524,7 +524,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -548,7 +548,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -567,10 +567,10 @@
         <v>18</v>
       </c>
       <c r="B19">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="C19">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -581,7 +581,7 @@
         <v>46</v>
       </c>
       <c r="C20">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -589,10 +589,10 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>99</v>
+        <v>22</v>
       </c>
       <c r="C21">
-        <v>3</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -600,10 +600,10 @@
         <v>21</v>
       </c>
       <c r="B22">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="C22">
-        <v>2</v>
+        <v>26</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -611,10 +611,10 @@
         <v>22</v>
       </c>
       <c r="B23">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -622,10 +622,10 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>330</v>
+        <v>200</v>
       </c>
       <c r="C24">
-        <v>33</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated reports for 6/17/25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="109">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/12/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/12/2025)</t>
+    <t>Adoptions (06/16/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/16/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -104,25 +104,40 @@
     <t>Review Date</t>
   </si>
   <si>
-    <t>A0058694543</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Cat Isolation 231, Cage 1</t>
-  </si>
-  <si>
-    <t>2025-06-17</t>
-  </si>
-  <si>
-    <t>A0058698177</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 05</t>
-  </si>
-  <si>
-    <t>A0058698188</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 02</t>
+    <t>A0058709950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Isolation 235, Cage 2</t>
+  </si>
+  <si>
+    <t>2025-06-19</t>
+  </si>
+  <si>
+    <t>A0058718824</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Treatment, 04</t>
+  </si>
+  <si>
+    <t>2025-06-20</t>
+  </si>
+  <si>
+    <t>A0058716138</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ICU, 01 - B</t>
+  </si>
+  <si>
+    <t>A0058706705</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 2</t>
+  </si>
+  <si>
+    <t>A0058716766</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Small Animals &amp; Exotics, Bird Cage 1</t>
   </si>
   <si>
     <t>AnimalNumber</t>
@@ -143,67 +158,76 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058089659</t>
-  </si>
-  <si>
-    <t>A0058579862</t>
-  </si>
-  <si>
-    <t>A0058653404</t>
-  </si>
-  <si>
-    <t>A0058653406</t>
-  </si>
-  <si>
-    <t>A0058655448</t>
-  </si>
-  <si>
-    <t>A0058661818</t>
-  </si>
-  <si>
-    <t>A0058676386</t>
-  </si>
-  <si>
-    <t>A0058688511</t>
-  </si>
-  <si>
-    <t>A0050951954</t>
-  </si>
-  <si>
-    <t>A0058622451</t>
-  </si>
-  <si>
-    <t>A0058640645</t>
-  </si>
-  <si>
-    <t>A0058694278</t>
-  </si>
-  <si>
-    <t>A0058694280</t>
-  </si>
-  <si>
-    <t>A0058694286</t>
-  </si>
-  <si>
-    <t>A0058696537</t>
-  </si>
-  <si>
-    <t>A0058696743</t>
-  </si>
-  <si>
-    <t>A0058696745</t>
-  </si>
-  <si>
-    <t>A0058696755</t>
-  </si>
-  <si>
-    <t>A0058696758</t>
-  </si>
-  <si>
-    <t>A0058697513</t>
-  </si>
-  <si>
-    <t>Rodent</t>
+    <t>A0058223085</t>
+  </si>
+  <si>
+    <t>A0058679860</t>
+  </si>
+  <si>
+    <t>A0058697050</t>
+  </si>
+  <si>
+    <t>A0058694957</t>
+  </si>
+  <si>
+    <t>A0058706029</t>
+  </si>
+  <si>
+    <t>A0058709460</t>
+  </si>
+  <si>
+    <t>A0058717573</t>
+  </si>
+  <si>
+    <t>A0058718209</t>
+  </si>
+  <si>
+    <t>A0058720454</t>
+  </si>
+  <si>
+    <t>A0058720471</t>
+  </si>
+  <si>
+    <t>A0058720491</t>
+  </si>
+  <si>
+    <t>A0058720528</t>
+  </si>
+  <si>
+    <t>A0058716081</t>
+  </si>
+  <si>
+    <t>A0058716470</t>
+  </si>
+  <si>
+    <t>A0058716471</t>
+  </si>
+  <si>
+    <t>A0058717101</t>
+  </si>
+  <si>
+    <t>A0058717112</t>
+  </si>
+  <si>
+    <t>A0058719464</t>
+  </si>
+  <si>
+    <t>A0058719477</t>
+  </si>
+  <si>
+    <t>A0058719482</t>
+  </si>
+  <si>
+    <t>A0058719488</t>
+  </si>
+  <si>
+    <t>A0058716736</t>
+  </si>
+  <si>
+    <t>Rabbit</t>
+  </si>
+  <si>
+    <t>Domestic (Cage) Bird</t>
   </si>
   <si>
     <t>Clinic</t>
@@ -212,100 +236,106 @@
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
+    <t>Seized / Custody</t>
+  </si>
+  <si>
+    <t>Stray</t>
+  </si>
+  <si>
+    <t>Transfer In</t>
+  </si>
+  <si>
+    <t>Retention</t>
+  </si>
+  <si>
+    <t>Euthanasia Request - OTC!</t>
+  </si>
+  <si>
+    <t>Cruelty</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>OTC</t>
+  </si>
+  <si>
+    <t>DOA</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>ACO or DCO in County</t>
+  </si>
+  <si>
+    <t>Clinic - Retention</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Seized – General</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Seized – Eviction</t>
+  </si>
+  <si>
+    <t>Seized – Police</t>
+  </si>
+  <si>
+    <t>Seized – Owner Died</t>
+  </si>
+  <si>
+    <t>Seized – Order Violation</t>
+  </si>
+  <si>
+    <t>Seized - Hoarding</t>
+  </si>
+  <si>
     <t>Return</t>
   </si>
   <si>
-    <t>Stray</t>
-  </si>
-  <si>
-    <t>Case - Outreach</t>
-  </si>
-  <si>
-    <t>Evaluation/Poss Adopt - OTC!</t>
-  </si>
-  <si>
-    <t>Euthanasia Request - OTC!</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Owned 30 Days or Less - OTC!</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>OTC</t>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>OTC - OS - SAFE</t>
+  </si>
+  <si>
+    <t>Clinic - Medical Treatment</t>
+  </si>
+  <si>
+    <t>Clinic - Stray</t>
+  </si>
+  <si>
+    <t>Clinic - Case Assistance</t>
   </si>
   <si>
     <t>Clinic - Case Assistance - Outreach</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Transfer In</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
-  </si>
-  <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
-    <t>Seized – General</t>
-  </si>
-  <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Seized – Eviction</t>
-  </si>
-  <si>
-    <t>Seized – Police</t>
-  </si>
-  <si>
-    <t>Seized – Owner Died</t>
-  </si>
-  <si>
-    <t>Seized – Order Violation</t>
-  </si>
-  <si>
-    <t>Seized - Hoarding</t>
-  </si>
-  <si>
-    <t>OTC - OS - SAFE</t>
-  </si>
-  <si>
-    <t>Clinic - Medical Treatment</t>
-  </si>
-  <si>
-    <t>Clinic - Stray</t>
-  </si>
-  <si>
-    <t>Clinic - Retention</t>
-  </si>
-  <si>
-    <t>Clinic - Case Assistance</t>
   </si>
   <si>
     <t>Clinic - Outreach</t>
@@ -688,7 +718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -708,7 +738,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -716,7 +746,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -732,7 +762,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>182</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -748,7 +778,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -772,7 +802,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>13</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -780,7 +810,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -788,7 +818,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -796,7 +826,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -804,7 +834,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -812,7 +842,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -820,7 +850,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -839,10 +869,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C20">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -850,7 +880,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C21">
         <v>19</v>
@@ -861,10 +891,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="C22">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -872,10 +902,10 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C23">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -886,7 +916,7 @@
         <v>0</v>
       </c>
       <c r="C24">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -894,10 +924,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="C25">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -930,188 +960,219 @@
         <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" t="s">
         <v>34</v>
       </c>
-      <c r="B30" t="s">
-        <v>35</v>
-      </c>
-      <c r="C30" t="s">
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="B33" s="1" t="s">
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" t="s">
+        <v>40</v>
+      </c>
+      <c r="C32" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B35" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C35" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
       </c>
       <c r="C36">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>80</v>
+        <v>85</v>
+      </c>
+      <c r="B38">
+        <v>3</v>
+      </c>
+      <c r="C38">
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>82</v>
+        <v>87</v>
+      </c>
+      <c r="B40">
+        <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>85</v>
+        <v>86</v>
+      </c>
+      <c r="C43">
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>65</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
-      </c>
-      <c r="C50">
-        <v>2</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>66</v>
-      </c>
-      <c r="B51">
-        <v>12</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>75</v>
-      </c>
-      <c r="C52">
-        <v>1</v>
-      </c>
-      <c r="D52">
-        <v>2</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>92</v>
+        <v>74</v>
+      </c>
+      <c r="B53">
+        <v>5</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>74</v>
-      </c>
-      <c r="B58">
+        <v>84</v>
+      </c>
+      <c r="C58">
+        <v>1</v>
+      </c>
+      <c r="D58">
         <v>2</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>98</v>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1121,487 +1182,527 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C2" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D2" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="F2" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C3" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="F3" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="C4" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="C5" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="F5" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D6" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="F7" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
       </c>
       <c r="C8" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D8" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="F8" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="F9" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
       </c>
       <c r="C12" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D12" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="F13" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E14" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D15" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E15" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F15" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
         <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E16" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="F16" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="C17" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E17" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F17" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
       <c r="C18" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D18" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E18" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F18" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
         <v>20</v>
       </c>
       <c r="C19" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D19" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E19" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="F19" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E20" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F20" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D21" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E21" t="s">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="F21" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D22" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F22" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="B23" t="s">
         <v>20</v>
       </c>
       <c r="C23" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D23" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F23" t="s">
-        <v>66</v>
+        <v>87</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="3">
-        <v>45820</v>
+        <v>45824</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="F24" t="s">
-        <v>66</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="3">
+        <v>45824</v>
+      </c>
+      <c r="D25" t="s">
+        <v>75</v>
+      </c>
+      <c r="E25" t="s">
+        <v>83</v>
+      </c>
+      <c r="F25" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>68</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="3">
+        <v>45824</v>
+      </c>
+      <c r="D26" t="s">
+        <v>75</v>
+      </c>
+      <c r="E26" t="s">
+        <v>83</v>
+      </c>
+      <c r="F26" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 6.18.25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="101">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/16/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/16/2025)</t>
+    <t>Adoptions (06/17/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/17/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -122,18 +122,21 @@
     <t>2025-06-20</t>
   </si>
   <si>
-    <t>A0058716138</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 01 - B</t>
-  </si>
-  <si>
     <t>A0058706705</t>
   </si>
   <si>
     <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 2</t>
   </si>
   <si>
+    <t>A0058727432</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 1</t>
+  </si>
+  <si>
+    <t>2025-06-24</t>
+  </si>
+  <si>
     <t>A0058716766</t>
   </si>
   <si>
@@ -158,76 +161,49 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058223085</t>
-  </si>
-  <si>
-    <t>A0058679860</t>
-  </si>
-  <si>
-    <t>A0058697050</t>
-  </si>
-  <si>
-    <t>A0058694957</t>
-  </si>
-  <si>
-    <t>A0058706029</t>
-  </si>
-  <si>
-    <t>A0058709460</t>
-  </si>
-  <si>
-    <t>A0058717573</t>
+    <t>A0058073288</t>
+  </si>
+  <si>
+    <t>A0058671143</t>
+  </si>
+  <si>
+    <t>A0058671146</t>
+  </si>
+  <si>
+    <t>A0058671149</t>
+  </si>
+  <si>
+    <t>A0058671153</t>
+  </si>
+  <si>
+    <t>A0058705115</t>
   </si>
   <si>
     <t>A0058718209</t>
   </si>
   <si>
-    <t>A0058720454</t>
-  </si>
-  <si>
-    <t>A0058720471</t>
-  </si>
-  <si>
-    <t>A0058720491</t>
-  </si>
-  <si>
-    <t>A0058720528</t>
-  </si>
-  <si>
-    <t>A0058716081</t>
-  </si>
-  <si>
-    <t>A0058716470</t>
-  </si>
-  <si>
-    <t>A0058716471</t>
-  </si>
-  <si>
-    <t>A0058717101</t>
-  </si>
-  <si>
-    <t>A0058717112</t>
-  </si>
-  <si>
-    <t>A0058719464</t>
-  </si>
-  <si>
-    <t>A0058719477</t>
-  </si>
-  <si>
-    <t>A0058719482</t>
-  </si>
-  <si>
-    <t>A0058719488</t>
-  </si>
-  <si>
-    <t>A0058716736</t>
-  </si>
-  <si>
-    <t>Rabbit</t>
-  </si>
-  <si>
-    <t>Domestic (Cage) Bird</t>
+    <t>A0058723929</t>
+  </si>
+  <si>
+    <t>A0058728965</t>
+  </si>
+  <si>
+    <t>A0058726103</t>
+  </si>
+  <si>
+    <t>A0058702607</t>
+  </si>
+  <si>
+    <t>A0058728323</t>
+  </si>
+  <si>
+    <t>A0058728669</t>
+  </si>
+  <si>
+    <t>Farm Type Fowl</t>
+  </si>
+  <si>
+    <t>Rodent</t>
   </si>
   <si>
     <t>Clinic</t>
@@ -242,94 +218,94 @@
     <t>Stray</t>
   </si>
   <si>
+    <t>Medical Treatment</t>
+  </si>
+  <si>
+    <t>OTC</t>
+  </si>
+  <si>
+    <t>Euthanasia Request - OTC!</t>
+  </si>
+  <si>
+    <t>DOA</t>
+  </si>
+  <si>
+    <t>Evaluation/Poss Adopt - OTC!</t>
+  </si>
+  <si>
+    <t>Cruelty</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Clinic - Medical Treatment</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
     <t>Transfer In</t>
   </si>
   <si>
-    <t>Retention</t>
-  </si>
-  <si>
-    <t>Euthanasia Request - OTC!</t>
-  </si>
-  <si>
-    <t>Cruelty</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>OTC</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>ACO or DCO in County</t>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Seized – General</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Seized – Eviction</t>
+  </si>
+  <si>
+    <t>Seized – Police</t>
+  </si>
+  <si>
+    <t>Seized – Owner Died</t>
+  </si>
+  <si>
+    <t>Seized – Order Violation</t>
+  </si>
+  <si>
+    <t>Seized - Hoarding</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>OTC - OS - SAFE</t>
+  </si>
+  <si>
+    <t>Clinic - Stray</t>
   </si>
   <si>
     <t>Clinic - Retention</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
-  </si>
-  <si>
-    <t>Seized – General</t>
-  </si>
-  <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Seized – Eviction</t>
-  </si>
-  <si>
-    <t>Seized – Police</t>
-  </si>
-  <si>
-    <t>Seized – Owner Died</t>
-  </si>
-  <si>
-    <t>Seized – Order Violation</t>
-  </si>
-  <si>
-    <t>Seized - Hoarding</t>
-  </si>
-  <si>
-    <t>Return</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
-    <t>OTC - OS - SAFE</t>
-  </si>
-  <si>
-    <t>Clinic - Medical Treatment</t>
-  </si>
-  <si>
-    <t>Clinic - Stray</t>
   </si>
   <si>
     <t>Clinic - Case Assistance</t>
@@ -738,7 +714,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>19</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -762,7 +738,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -778,7 +754,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -802,7 +778,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -818,7 +794,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -826,7 +802,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -834,7 +810,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>11</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -850,7 +826,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -869,7 +845,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C20">
         <v>28</v>
@@ -880,7 +856,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C21">
         <v>19</v>
@@ -891,10 +867,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C22">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -927,7 +903,7 @@
         <v>145</v>
       </c>
       <c r="C25">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -971,7 +947,7 @@
         <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -982,15 +958,15 @@
         <v>38</v>
       </c>
       <c r="C31" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C32" t="s">
         <v>34</v>
@@ -998,7 +974,7 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>20</v>
@@ -1012,26 +988,20 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>75</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
-      </c>
-      <c r="C36">
-        <v>1</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>81</v>
+        <v>70</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>85</v>
-      </c>
-      <c r="B38">
-        <v>3</v>
+        <v>77</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -1039,86 +1009,86 @@
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B40">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="C43">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B53">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D53">
         <v>1</v>
@@ -1126,53 +1096,56 @@
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>101</v>
+        <v>76</v>
+      </c>
+      <c r="B54">
+        <v>4</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>103</v>
+        <v>75</v>
+      </c>
+      <c r="C56">
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>84</v>
-      </c>
-      <c r="C58">
-        <v>1</v>
-      </c>
-      <c r="D58">
-        <v>2</v>
+        <v>96</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1182,267 +1155,267 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="F2" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E3" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" t="s">
         <v>76</v>
-      </c>
-      <c r="F3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D4" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" t="s">
         <v>76</v>
-      </c>
-      <c r="F4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E5" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="F6" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F7" t="s">
         <v>77</v>
-      </c>
-      <c r="F7" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E8" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="F8" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D9" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E9" t="s">
+        <v>69</v>
+      </c>
+      <c r="F9" t="s">
         <v>77</v>
-      </c>
-      <c r="F9" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="C10" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D10" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="E10" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="F10" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D11" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" t="s">
         <v>78</v>
-      </c>
-      <c r="F11" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E12" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="C13" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D13" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E13" t="s">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="F13" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -1453,16 +1426,16 @@
         <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D14" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="E14" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="F14" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -1473,236 +1446,16 @@
         <v>20</v>
       </c>
       <c r="C15" s="3">
-        <v>45824</v>
+        <v>45825</v>
       </c>
       <c r="D15" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" t="s">
         <v>74</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>79</v>
-      </c>
-      <c r="F15" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
-        <v>61</v>
-      </c>
-      <c r="B16" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D16" t="s">
-        <v>74</v>
-      </c>
-      <c r="E16" t="s">
-        <v>79</v>
-      </c>
-      <c r="F16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6">
-      <c r="A17" t="s">
-        <v>39</v>
-      </c>
-      <c r="B17" t="s">
-        <v>70</v>
-      </c>
-      <c r="C17" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D17" t="s">
-        <v>74</v>
-      </c>
-      <c r="E17" t="s">
-        <v>80</v>
-      </c>
-      <c r="F17" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6">
-      <c r="A18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B18" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D18" t="s">
-        <v>74</v>
-      </c>
-      <c r="E18" t="s">
-        <v>81</v>
-      </c>
-      <c r="F18" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" t="s">
-        <v>63</v>
-      </c>
-      <c r="B19" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D19" t="s">
-        <v>74</v>
-      </c>
-      <c r="E19" t="s">
-        <v>81</v>
-      </c>
-      <c r="F19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" t="s">
-        <v>20</v>
-      </c>
-      <c r="C20" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D20" t="s">
-        <v>74</v>
-      </c>
-      <c r="E20" t="s">
-        <v>82</v>
-      </c>
-      <c r="F20" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
-      <c r="A21" t="s">
-        <v>64</v>
-      </c>
-      <c r="B21" t="s">
-        <v>20</v>
-      </c>
-      <c r="C21" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D21" t="s">
-        <v>74</v>
-      </c>
-      <c r="E21" t="s">
-        <v>82</v>
-      </c>
-      <c r="F21" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6">
-      <c r="A22" t="s">
-        <v>65</v>
-      </c>
-      <c r="B22" t="s">
-        <v>20</v>
-      </c>
-      <c r="C22" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D22" t="s">
-        <v>74</v>
-      </c>
-      <c r="E22" t="s">
-        <v>82</v>
-      </c>
-      <c r="F22" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6">
-      <c r="A23" t="s">
-        <v>66</v>
-      </c>
-      <c r="B23" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D23" t="s">
-        <v>74</v>
-      </c>
-      <c r="E23" t="s">
-        <v>82</v>
-      </c>
-      <c r="F23" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6">
-      <c r="A24" t="s">
-        <v>67</v>
-      </c>
-      <c r="B24" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D24" t="s">
-        <v>74</v>
-      </c>
-      <c r="E24" t="s">
-        <v>82</v>
-      </c>
-      <c r="F24" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
-      <c r="A25" t="s">
-        <v>35</v>
-      </c>
-      <c r="B25" t="s">
-        <v>20</v>
-      </c>
-      <c r="C25" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D25" t="s">
-        <v>75</v>
-      </c>
-      <c r="E25" t="s">
-        <v>83</v>
-      </c>
-      <c r="F25" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6">
-      <c r="A26" t="s">
-        <v>68</v>
-      </c>
-      <c r="B26" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="3">
-        <v>45824</v>
-      </c>
-      <c r="D26" t="s">
-        <v>75</v>
-      </c>
-      <c r="E26" t="s">
-        <v>83</v>
-      </c>
-      <c r="F26" t="s">
-        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 6.19.25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="98">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/17/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/17/2025)</t>
+    <t>Adoptions (06/18/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/18/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -104,15 +104,6 @@
     <t>Review Date</t>
   </si>
   <si>
-    <t>A0058709950</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Cat Isolation 235, Cage 2</t>
-  </si>
-  <si>
-    <t>2025-06-19</t>
-  </si>
-  <si>
     <t>A0058718824</t>
   </si>
   <si>
@@ -122,12 +113,6 @@
     <t>2025-06-20</t>
   </si>
   <si>
-    <t>A0058706705</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 2</t>
-  </si>
-  <si>
     <t>A0058727432</t>
   </si>
   <si>
@@ -161,52 +146,61 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058073288</t>
-  </si>
-  <si>
-    <t>A0058671143</t>
-  </si>
-  <si>
-    <t>A0058671146</t>
-  </si>
-  <si>
-    <t>A0058671149</t>
-  </si>
-  <si>
-    <t>A0058671153</t>
-  </si>
-  <si>
-    <t>A0058705115</t>
-  </si>
-  <si>
-    <t>A0058718209</t>
-  </si>
-  <si>
-    <t>A0058723929</t>
-  </si>
-  <si>
-    <t>A0058728965</t>
-  </si>
-  <si>
-    <t>A0058726103</t>
-  </si>
-  <si>
-    <t>A0058702607</t>
-  </si>
-  <si>
-    <t>A0058728323</t>
-  </si>
-  <si>
-    <t>A0058728669</t>
-  </si>
-  <si>
-    <t>Farm Type Fowl</t>
-  </si>
-  <si>
-    <t>Rodent</t>
-  </si>
-  <si>
-    <t>Clinic</t>
+    <t>A0058736922</t>
+  </si>
+  <si>
+    <t>A0058737339</t>
+  </si>
+  <si>
+    <t>A0058733210</t>
+  </si>
+  <si>
+    <t>A0058737658</t>
+  </si>
+  <si>
+    <t>A0058732745</t>
+  </si>
+  <si>
+    <t>A0058733446</t>
+  </si>
+  <si>
+    <t>A0058736662</t>
+  </si>
+  <si>
+    <t>A0058738023</t>
+  </si>
+  <si>
+    <t>A0058718199</t>
+  </si>
+  <si>
+    <t>A0058718216</t>
+  </si>
+  <si>
+    <t>A0058718227</t>
+  </si>
+  <si>
+    <t>A0058718231</t>
+  </si>
+  <si>
+    <t>A0058718238</t>
+  </si>
+  <si>
+    <t>A0058718243</t>
+  </si>
+  <si>
+    <t>A0058718252</t>
+  </si>
+  <si>
+    <t>A0058718268</t>
+  </si>
+  <si>
+    <t>A0058718282</t>
+  </si>
+  <si>
+    <t>A0058718292</t>
+  </si>
+  <si>
+    <t>A0058718303</t>
   </si>
   <si>
     <t>Owner/Guardian Surrender</t>
@@ -218,88 +212,85 @@
     <t>Stray</t>
   </si>
   <si>
-    <t>Medical Treatment</t>
-  </si>
-  <si>
-    <t>OTC</t>
+    <t>Transfer In</t>
   </si>
   <si>
     <t>Euthanasia Request - OTC!</t>
   </si>
   <si>
+    <t>Evaluation/Poss Adopt - FIELD!</t>
+  </si>
+  <si>
+    <t>Signed Over</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Rescue Group out of Coalition</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
     <t>DOA</t>
   </si>
   <si>
-    <t>Evaluation/Poss Adopt - OTC!</t>
-  </si>
-  <si>
-    <t>Cruelty</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>Field</t>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Seized – General</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
+    <t>Seized – Eviction</t>
+  </si>
+  <si>
+    <t>Seized – Police</t>
+  </si>
+  <si>
+    <t>Seized – Owner Died</t>
+  </si>
+  <si>
+    <t>Seized – Order Violation</t>
+  </si>
+  <si>
+    <t>Seized - Hoarding</t>
+  </si>
+  <si>
+    <t>Return</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>OTC - OS - SAFE</t>
   </si>
   <si>
     <t>Clinic - Medical Treatment</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Transfer In</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
-  </si>
-  <si>
-    <t>Seized – General</t>
-  </si>
-  <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Seized – Eviction</t>
-  </si>
-  <si>
-    <t>Seized – Police</t>
-  </si>
-  <si>
-    <t>Seized – Owner Died</t>
-  </si>
-  <si>
-    <t>Seized – Order Violation</t>
-  </si>
-  <si>
-    <t>Seized - Hoarding</t>
-  </si>
-  <si>
-    <t>Return</t>
-  </si>
-  <si>
-    <t>OTC - OS - SAFE</t>
   </si>
   <si>
     <t>Clinic - Stray</t>
@@ -694,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -714,7 +705,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -722,7 +713,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -738,7 +729,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>188</v>
+        <v>192</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -754,7 +745,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -778,7 +769,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>14</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -794,7 +785,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -802,7 +793,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -810,7 +801,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -826,7 +817,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -845,10 +836,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C20">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -856,7 +847,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C21">
         <v>19</v>
@@ -867,10 +858,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C22">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -878,10 +869,10 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C23">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -889,7 +880,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -900,10 +891,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C25">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -950,202 +941,171 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:3">
-      <c r="A31" t="s">
-        <v>37</v>
-      </c>
-      <c r="B31" t="s">
-        <v>38</v>
-      </c>
-      <c r="C31" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" t="s">
-        <v>40</v>
-      </c>
-      <c r="B32" t="s">
-        <v>41</v>
-      </c>
-      <c r="C32" t="s">
-        <v>34</v>
+    <row r="33" spans="1:4">
+      <c r="A33" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34">
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>23</v>
+      <c r="A35" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>81</v>
+        <v>72</v>
+      </c>
+      <c r="B36">
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>70</v>
-      </c>
-      <c r="B37">
-        <v>1</v>
+        <v>78</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>77</v>
-      </c>
-      <c r="C38">
-        <v>2</v>
+        <v>75</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>82</v>
+        <v>73</v>
+      </c>
+      <c r="B39">
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
         <v>79</v>
       </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>78</v>
-      </c>
-      <c r="C43">
-        <v>1</v>
+        <v>82</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>74</v>
+      </c>
+      <c r="C44">
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>64</v>
+      </c>
+      <c r="B51">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
-      <c r="A49" t="s">
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
-      <c r="A50" t="s">
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
-      <c r="A51" t="s">
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
-      <c r="A52" t="s">
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
-      <c r="A53" t="s">
-        <v>66</v>
-      </c>
-      <c r="B53">
-        <v>2</v>
-      </c>
-      <c r="D53">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4">
-      <c r="A54" t="s">
-        <v>76</v>
-      </c>
-      <c r="B54">
-        <v>4</v>
-      </c>
-      <c r="D54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4">
-      <c r="A55" t="s">
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
-      <c r="A56" t="s">
-        <v>75</v>
-      </c>
-      <c r="C56">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4">
-      <c r="A57" t="s">
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
-      <c r="A58" t="s">
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
-      <c r="A59" t="s">
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
         <v>97</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4">
-      <c r="A60" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4">
-      <c r="A61" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="A62" t="s">
-        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1155,138 +1115,138 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
       </c>
       <c r="C3" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E4" t="s">
         <v>68</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E5" t="s">
         <v>68</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D6" t="s">
         <v>64</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D7" t="s">
         <v>64</v>
@@ -1295,167 +1255,267 @@
         <v>69</v>
       </c>
       <c r="F7" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D8" t="s">
         <v>64</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D9" t="s">
         <v>64</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F9" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E10" t="s">
         <v>71</v>
       </c>
       <c r="F10" t="s">
-        <v>76</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D11" t="s">
         <v>65</v>
       </c>
       <c r="E11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>54</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E13" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C14" s="3">
-        <v>45825</v>
+        <v>45826</v>
       </c>
       <c r="D14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="3">
+        <v>45826</v>
+      </c>
+      <c r="D15" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" t="s">
+        <v>71</v>
+      </c>
+      <c r="F15" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="3">
+        <v>45826</v>
+      </c>
+      <c r="D16" t="s">
+        <v>65</v>
+      </c>
+      <c r="E16" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>58</v>
+      </c>
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="3">
+        <v>45826</v>
+      </c>
+      <c r="D17" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" t="s">
+        <v>71</v>
+      </c>
+      <c r="F17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="3">
+        <v>45826</v>
+      </c>
+      <c r="D18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18" t="s">
+        <v>71</v>
+      </c>
+      <c r="F18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
         <v>60</v>
       </c>
-      <c r="B15" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="3">
-        <v>45825</v>
-      </c>
-      <c r="D15" t="s">
-        <v>66</v>
-      </c>
-      <c r="E15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F15" t="s">
-        <v>79</v>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="3">
+        <v>45826</v>
+      </c>
+      <c r="D19" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" t="s">
+        <v>71</v>
+      </c>
+      <c r="F19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="3">
+        <v>45826</v>
+      </c>
+      <c r="D20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" t="s">
+        <v>71</v>
+      </c>
+      <c r="F20" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 6/20/25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="93">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/18/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/18/2025)</t>
+    <t>Adoptions (06/19/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/19/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -104,13 +104,13 @@
     <t>Review Date</t>
   </si>
   <si>
-    <t>A0058718824</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Cat Treatment, 04</t>
-  </si>
-  <si>
-    <t>2025-06-20</t>
+    <t>A0058734302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Isolation 234, Cage 2</t>
+  </si>
+  <si>
+    <t>2025-06-24</t>
   </si>
   <si>
     <t>A0058727432</t>
@@ -119,15 +119,6 @@
     <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 1</t>
   </si>
   <si>
-    <t>2025-06-24</t>
-  </si>
-  <si>
-    <t>A0058716766</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Small Animals &amp; Exotics, Bird Cage 1</t>
-  </si>
-  <si>
     <t>AnimalNumber</t>
   </si>
   <si>
@@ -146,67 +137,61 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058736922</t>
-  </si>
-  <si>
-    <t>A0058737339</t>
-  </si>
-  <si>
-    <t>A0058733210</t>
-  </si>
-  <si>
-    <t>A0058737658</t>
-  </si>
-  <si>
-    <t>A0058732745</t>
-  </si>
-  <si>
-    <t>A0058733446</t>
-  </si>
-  <si>
-    <t>A0058736662</t>
-  </si>
-  <si>
-    <t>A0058738023</t>
-  </si>
-  <si>
-    <t>A0058718199</t>
-  </si>
-  <si>
-    <t>A0058718216</t>
-  </si>
-  <si>
-    <t>A0058718227</t>
-  </si>
-  <si>
-    <t>A0058718231</t>
-  </si>
-  <si>
-    <t>A0058718238</t>
-  </si>
-  <si>
-    <t>A0058718243</t>
-  </si>
-  <si>
-    <t>A0058718252</t>
-  </si>
-  <si>
-    <t>A0058718268</t>
-  </si>
-  <si>
-    <t>A0058718282</t>
-  </si>
-  <si>
-    <t>A0058718292</t>
-  </si>
-  <si>
-    <t>A0058718303</t>
+    <t>A0051151112</t>
+  </si>
+  <si>
+    <t>A0058737688</t>
+  </si>
+  <si>
+    <t>A0058744626</t>
+  </si>
+  <si>
+    <t>A0058744628</t>
+  </si>
+  <si>
+    <t>A0058744631</t>
+  </si>
+  <si>
+    <t>A0058744636</t>
+  </si>
+  <si>
+    <t>A0058744640</t>
+  </si>
+  <si>
+    <t>A0046108202</t>
+  </si>
+  <si>
+    <t>A0050275902</t>
+  </si>
+  <si>
+    <t>A0052271961</t>
+  </si>
+  <si>
+    <t>A0058741355</t>
+  </si>
+  <si>
+    <t>A0058741358</t>
+  </si>
+  <si>
+    <t>A0058741713</t>
+  </si>
+  <si>
+    <t>A0058741830</t>
+  </si>
+  <si>
+    <t>A0058742495</t>
+  </si>
+  <si>
+    <t>A0058743361</t>
+  </si>
+  <si>
+    <t>A0058690617</t>
   </si>
   <si>
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
-    <t>Seized / Custody</t>
+    <t>Return</t>
   </si>
   <si>
     <t>Stray</t>
@@ -221,16 +206,22 @@
     <t>Evaluation/Poss Adopt - FIELD!</t>
   </si>
   <si>
-    <t>Signed Over</t>
+    <t>Owned More than 30 Days - OTC!</t>
+  </si>
+  <si>
+    <t>OTC</t>
   </si>
   <si>
     <t>No Hold</t>
   </si>
   <si>
+    <t>DOA</t>
+  </si>
+  <si>
     <t>Field</t>
   </si>
   <si>
-    <t>Rescue Group out of Coalition</t>
+    <t>SPCA - Other Counties</t>
   </si>
   <si>
     <t>Euthanasia Request</t>
@@ -239,33 +230,30 @@
     <t>Field – OS</t>
   </si>
   <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Seized – General</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
     <t>Seized – Signed over</t>
   </si>
   <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
-  </si>
-  <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
-    <t>Seized – General</t>
-  </si>
-  <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
     <t>Seized – Eviction</t>
   </si>
   <si>
@@ -279,9 +267,6 @@
   </si>
   <si>
     <t>Seized - Hoarding</t>
-  </si>
-  <si>
-    <t>Return</t>
   </si>
   <si>
     <t>OTC – OS</t>
@@ -685,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D59"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -705,7 +690,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -713,7 +698,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -729,7 +714,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>192</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -745,7 +730,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -769,7 +754,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -801,7 +786,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -812,15 +797,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:4">
       <c r="A17" t="s">
         <v>16</v>
       </c>
       <c r="B17">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -831,7 +816,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:4">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -842,7 +827,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:4">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -850,32 +835,32 @@
         <v>36</v>
       </c>
       <c r="C21">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" t="s">
         <v>22</v>
       </c>
       <c r="B22">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="C22">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" t="s">
         <v>23</v>
       </c>
       <c r="B23">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C23">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:4">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -886,18 +871,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:3">
+    <row r="25" spans="1:4">
       <c r="A25" t="s">
         <v>25</v>
       </c>
       <c r="B25">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="C25">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
@@ -908,7 +893,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:3">
+    <row r="28" spans="1:4">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -919,7 +904,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:4">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -927,185 +912,180 @@
         <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>35</v>
-      </c>
-      <c r="B30" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="1" t="s">
+    <row r="32" spans="1:4">
+      <c r="A32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>60</v>
+      </c>
+      <c r="C33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>69</v>
+      </c>
+      <c r="B35">
+        <v>1</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
         <v>76</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="36" spans="1:4">
-      <c r="A36" t="s">
-        <v>72</v>
-      </c>
-      <c r="B36">
+    <row r="43" spans="1:3">
+      <c r="A43" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" t="s">
+        <v>58</v>
+      </c>
+      <c r="B49">
+        <v>2</v>
+      </c>
+      <c r="C49">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4">
-      <c r="A37" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" t="s">
-        <v>75</v>
-      </c>
-      <c r="B38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" t="s">
-        <v>73</v>
-      </c>
-      <c r="B39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
-      <c r="A44" t="s">
-        <v>74</v>
-      </c>
-      <c r="C44">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4">
-      <c r="A45" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4">
-      <c r="A46" t="s">
+    <row r="50" spans="1:3">
+      <c r="A50" t="s">
+        <v>59</v>
+      </c>
+      <c r="B50">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="47" spans="1:4">
-      <c r="A47" t="s">
+    <row r="52" spans="1:3">
+      <c r="A52" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
-      <c r="A48" t="s">
+    <row r="53" spans="1:3">
+      <c r="A53" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
-      <c r="A49" t="s">
+    <row r="54" spans="1:3">
+      <c r="A54" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
-      <c r="A50" t="s">
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
-      <c r="A51" t="s">
-        <v>64</v>
-      </c>
-      <c r="B51">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2">
-      <c r="A52" t="s">
+    <row r="56" spans="1:3">
+      <c r="A56" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
-      <c r="A53" t="s">
+    <row r="57" spans="1:3">
+      <c r="A57" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
-      <c r="A54" t="s">
+    <row r="58" spans="1:3">
+      <c r="A58" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
-      <c r="A55" t="s">
+    <row r="59" spans="1:3">
+      <c r="A59" t="s">
         <v>92</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2">
-      <c r="A56" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2">
-      <c r="A57" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2">
-      <c r="A58" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2">
-      <c r="A59" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2">
-      <c r="A60" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1115,407 +1095,387 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D2" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
       </c>
       <c r="C3" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D3" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D4" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="F5" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D6" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="F6" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
       </c>
       <c r="C7" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="F7" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D8" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="F8" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>75</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D10" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E10" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="F10" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="F11" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C12" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D12" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E12" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D13" t="s">
+        <v>59</v>
+      </c>
+      <c r="E13" t="s">
         <v>65</v>
       </c>
-      <c r="E13" t="s">
-        <v>71</v>
-      </c>
       <c r="F13" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D14" t="s">
+        <v>59</v>
+      </c>
+      <c r="E14" t="s">
         <v>65</v>
       </c>
-      <c r="E14" t="s">
-        <v>71</v>
-      </c>
       <c r="F14" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D15" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E15" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="F15" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D16" t="s">
+        <v>59</v>
+      </c>
+      <c r="E16" t="s">
         <v>65</v>
       </c>
-      <c r="E16" t="s">
-        <v>71</v>
-      </c>
       <c r="F16" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E17" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="F17" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="3">
+        <v>45827</v>
+      </c>
+      <c r="D18" t="s">
         <v>59</v>
       </c>
-      <c r="B18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="3">
-        <v>45826</v>
-      </c>
-      <c r="D18" t="s">
-        <v>65</v>
-      </c>
       <c r="E18" t="s">
+        <v>67</v>
+      </c>
+      <c r="F18" t="s">
         <v>71</v>
-      </c>
-      <c r="F18" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B19" t="s">
         <v>21</v>
       </c>
       <c r="C19" s="3">
-        <v>45826</v>
+        <v>45827</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="E19" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F19" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C20" s="3">
-        <v>45826</v>
-      </c>
-      <c r="D20" t="s">
-        <v>65</v>
-      </c>
-      <c r="E20" t="s">
-        <v>71</v>
-      </c>
-      <c r="F20" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 6/23/25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="122">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/19/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/19/2025)</t>
+    <t>Adoptions (06/20/2025, 6/21/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/20/2025, 6/21/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -104,6 +104,15 @@
     <t>Review Date</t>
   </si>
   <si>
+    <t>A0058695418</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Adoption Condo Rooms, Rabbitat 1</t>
+  </si>
+  <si>
+    <t>2025-06-26</t>
+  </si>
+  <si>
     <t>A0058734302</t>
   </si>
   <si>
@@ -113,6 +122,15 @@
     <t>2025-06-24</t>
   </si>
   <si>
+    <t>A0035002298</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ICU, 01 - B</t>
+  </si>
+  <si>
+    <t>No Review Date</t>
+  </si>
+  <si>
     <t>A0058727432</t>
   </si>
   <si>
@@ -137,55 +155,112 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0051151112</t>
-  </si>
-  <si>
-    <t>A0058737688</t>
-  </si>
-  <si>
-    <t>A0058744626</t>
-  </si>
-  <si>
-    <t>A0058744628</t>
-  </si>
-  <si>
-    <t>A0058744631</t>
-  </si>
-  <si>
-    <t>A0058744636</t>
-  </si>
-  <si>
-    <t>A0058744640</t>
-  </si>
-  <si>
-    <t>A0046108202</t>
-  </si>
-  <si>
-    <t>A0050275902</t>
-  </si>
-  <si>
-    <t>A0052271961</t>
-  </si>
-  <si>
-    <t>A0058741355</t>
-  </si>
-  <si>
-    <t>A0058741358</t>
-  </si>
-  <si>
-    <t>A0058741713</t>
-  </si>
-  <si>
-    <t>A0058741830</t>
-  </si>
-  <si>
-    <t>A0058742495</t>
-  </si>
-  <si>
-    <t>A0058743361</t>
-  </si>
-  <si>
-    <t>A0058690617</t>
+    <t>A0058581988</t>
+  </si>
+  <si>
+    <t>A0058727921</t>
+  </si>
+  <si>
+    <t>A0058729123</t>
+  </si>
+  <si>
+    <t>A0058748113</t>
+  </si>
+  <si>
+    <t>A0058748530</t>
+  </si>
+  <si>
+    <t>A0058748533</t>
+  </si>
+  <si>
+    <t>A0058748536</t>
+  </si>
+  <si>
+    <t>A0058748541</t>
+  </si>
+  <si>
+    <t>A0058748559</t>
+  </si>
+  <si>
+    <t>A0058748561</t>
+  </si>
+  <si>
+    <t>A0058748566</t>
+  </si>
+  <si>
+    <t>A0058748569</t>
+  </si>
+  <si>
+    <t>A0058748790</t>
+  </si>
+  <si>
+    <t>A0058748794</t>
+  </si>
+  <si>
+    <t>A0058749076</t>
+  </si>
+  <si>
+    <t>A0058752173</t>
+  </si>
+  <si>
+    <t>A0058755847</t>
+  </si>
+  <si>
+    <t>A0058757630</t>
+  </si>
+  <si>
+    <t>A0058757640</t>
+  </si>
+  <si>
+    <t>A0058758488</t>
+  </si>
+  <si>
+    <t>A0058622436</t>
+  </si>
+  <si>
+    <t>A0058753935</t>
+  </si>
+  <si>
+    <t>A0058753940</t>
+  </si>
+  <si>
+    <t>A0058753950</t>
+  </si>
+  <si>
+    <t>A0058753956</t>
+  </si>
+  <si>
+    <t>A0058753958</t>
+  </si>
+  <si>
+    <t>A0058753963</t>
+  </si>
+  <si>
+    <t>A0058753970</t>
+  </si>
+  <si>
+    <t>A0058753979</t>
+  </si>
+  <si>
+    <t>A0058753987</t>
+  </si>
+  <si>
+    <t>A0058747360</t>
+  </si>
+  <si>
+    <t>A0058747362</t>
+  </si>
+  <si>
+    <t>A0058755856</t>
+  </si>
+  <si>
+    <t>A0058755861</t>
+  </si>
+  <si>
+    <t>A0058757250</t>
+  </si>
+  <si>
+    <t>Rabbit</t>
   </si>
   <si>
     <t>Owner/Guardian Surrender</t>
@@ -194,51 +269,69 @@
     <t>Return</t>
   </si>
   <si>
+    <t>Seized / Custody</t>
+  </si>
+  <si>
     <t>Stray</t>
   </si>
   <si>
     <t>Transfer In</t>
   </si>
   <si>
+    <t>Evaluation/Poss Adopt - OTC!</t>
+  </si>
+  <si>
     <t>Euthanasia Request - OTC!</t>
   </si>
   <si>
     <t>Evaluation/Poss Adopt - FIELD!</t>
   </si>
   <si>
-    <t>Owned More than 30 Days - OTC!</t>
-  </si>
-  <si>
     <t>OTC</t>
   </si>
   <si>
+    <t>Euthanasia Request - FIELD!</t>
+  </si>
+  <si>
+    <t>Guardian Surrender - FIELD!</t>
+  </si>
+  <si>
+    <t>Owned 30 Days or Less - OTC!</t>
+  </si>
+  <si>
+    <t>Signed Over</t>
+  </si>
+  <si>
     <t>No Hold</t>
   </si>
   <si>
+    <t>Vet clinic</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
     <t>DOA</t>
   </si>
   <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>SPCA - Other Counties</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
     <t>Field – Stray</t>
   </si>
   <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
     <t>Seized – Abandoned</t>
   </si>
   <si>
@@ -251,9 +344,6 @@
     <t>Seized – Hospital</t>
   </si>
   <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
     <t>Seized – Eviction</t>
   </si>
   <si>
@@ -267,9 +357,6 @@
   </si>
   <si>
     <t>Seized - Hoarding</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
   </si>
   <si>
     <t>OTC - OS - SAFE</t>
@@ -670,7 +757,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -690,7 +777,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -698,7 +785,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -714,7 +801,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>199</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -730,7 +817,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -754,7 +841,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -770,7 +857,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -778,7 +865,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>14</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -794,18 +881,18 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
       <c r="B17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -816,18 +903,18 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
       <c r="B20">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C20">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -835,32 +922,32 @@
         <v>36</v>
       </c>
       <c r="C21">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
       <c r="B22">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C22">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>23</v>
       </c>
       <c r="B23">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C23">
         <v>25</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>24</v>
       </c>
@@ -871,18 +958,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
       <c r="B25">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C25">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
@@ -893,7 +980,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -904,7 +991,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -912,180 +999,217 @@
         <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B32" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B34" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C34" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D34" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>60</v>
-      </c>
-      <c r="C33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
+    <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="B35">
         <v>1</v>
       </c>
-      <c r="C35">
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
+      <c r="A37" t="s">
+        <v>98</v>
+      </c>
+      <c r="C37">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
+      <c r="A38" t="s">
+        <v>100</v>
+      </c>
+      <c r="C38">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
-      <c r="A37" t="s">
-        <v>71</v>
-      </c>
-      <c r="B37">
+    <row r="39" spans="1:4">
+      <c r="A39" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>99</v>
+      </c>
+      <c r="B40">
+        <v>3</v>
+      </c>
+      <c r="C40">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>101</v>
+      </c>
+      <c r="B45">
+        <v>6</v>
+      </c>
+      <c r="C45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
+      <c r="A48" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
+      <c r="A49" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
+      <c r="A50" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
+      <c r="A51" t="s">
+        <v>83</v>
+      </c>
+      <c r="C51">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
-      <c r="A38" t="s">
-        <v>70</v>
-      </c>
-      <c r="B38">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
-      <c r="A48" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
-      <c r="A49" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49">
-        <v>2</v>
-      </c>
-      <c r="C49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
-      <c r="A50" t="s">
-        <v>59</v>
-      </c>
-      <c r="B50">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
-      <c r="A51" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
+    <row r="52" spans="1:4">
       <c r="A52" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="53" spans="1:3">
+      <c r="B52">
+        <v>6</v>
+      </c>
+      <c r="D52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3">
+        <v>97</v>
+      </c>
+      <c r="B53">
+        <v>1</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+      <c r="D53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>92</v>
+        <v>119</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -1095,387 +1219,787 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>97</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="E3" t="s">
-        <v>61</v>
+        <v>88</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D4" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="E4" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="F4" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="E5" t="s">
-        <v>62</v>
+        <v>88</v>
       </c>
       <c r="F5" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="E6" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="F6" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="E7" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="F7" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C8" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>82</v>
       </c>
       <c r="E8" t="s">
-        <v>62</v>
+        <v>89</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D10" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="E10" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="E11" t="s">
-        <v>61</v>
+        <v>89</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D12" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="F12" t="s">
-        <v>59</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E13" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="F13" t="s">
-        <v>59</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D14" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E14" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="F14" t="s">
-        <v>59</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D15" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E15" t="s">
-        <v>64</v>
+        <v>89</v>
       </c>
       <c r="F15" t="s">
-        <v>59</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C16" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D16" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="F16" t="s">
-        <v>59</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="3">
-        <v>45827</v>
+        <v>45828</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E17" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="F17" t="s">
-        <v>59</v>
+        <v>97</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B18" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C18" s="3">
-        <v>45827</v>
+        <v>45829</v>
       </c>
       <c r="D18" t="s">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="F18" t="s">
-        <v>71</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="B19" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="3">
+        <v>45829</v>
+      </c>
+      <c r="D19" t="s">
+        <v>82</v>
+      </c>
+      <c r="E19" t="s">
+        <v>87</v>
+      </c>
+      <c r="F19" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>81</v>
+      </c>
+      <c r="C20" s="3">
+        <v>45829</v>
+      </c>
+      <c r="D20" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="3">
+        <v>45829</v>
+      </c>
+      <c r="D21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E21" t="s">
+        <v>92</v>
+      </c>
+      <c r="F21" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="3">
-        <v>45827</v>
-      </c>
-      <c r="D19" t="s">
-        <v>60</v>
-      </c>
-      <c r="E19" t="s">
+      <c r="C22" s="3">
+        <v>45829</v>
+      </c>
+      <c r="D22" t="s">
+        <v>83</v>
+      </c>
+      <c r="E22" t="s">
+        <v>93</v>
+      </c>
+      <c r="F22" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D23" t="s">
+        <v>84</v>
+      </c>
+      <c r="E23" t="s">
+        <v>94</v>
+      </c>
+      <c r="F23" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
         <v>68</v>
       </c>
-      <c r="F19" t="s">
-        <v>60</v>
+      <c r="B24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D24" t="s">
+        <v>84</v>
+      </c>
+      <c r="E24" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D25" t="s">
+        <v>84</v>
+      </c>
+      <c r="E25" t="s">
+        <v>94</v>
+      </c>
+      <c r="F25" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D26" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26" t="s">
+        <v>94</v>
+      </c>
+      <c r="F26" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D27" t="s">
+        <v>84</v>
+      </c>
+      <c r="E27" t="s">
+        <v>94</v>
+      </c>
+      <c r="F27" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>72</v>
+      </c>
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28" t="s">
+        <v>94</v>
+      </c>
+      <c r="F28" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D29" t="s">
+        <v>84</v>
+      </c>
+      <c r="E29" t="s">
+        <v>94</v>
+      </c>
+      <c r="F29" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>74</v>
+      </c>
+      <c r="B30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D30" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" t="s">
+        <v>94</v>
+      </c>
+      <c r="F30" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D31" t="s">
+        <v>84</v>
+      </c>
+      <c r="E31" t="s">
+        <v>94</v>
+      </c>
+      <c r="F31" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D32" t="s">
+        <v>85</v>
+      </c>
+      <c r="E32" t="s">
+        <v>90</v>
+      </c>
+      <c r="F32" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>35</v>
+      </c>
+      <c r="B33" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D33" t="s">
+        <v>85</v>
+      </c>
+      <c r="E33" t="s">
+        <v>90</v>
+      </c>
+      <c r="F33" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" t="s">
+        <v>81</v>
+      </c>
+      <c r="C34" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D34" t="s">
+        <v>85</v>
+      </c>
+      <c r="E34" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>76</v>
+      </c>
+      <c r="B35" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D35" t="s">
+        <v>85</v>
+      </c>
+      <c r="E35" t="s">
+        <v>95</v>
+      </c>
+      <c r="F35" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>77</v>
+      </c>
+      <c r="B36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="3">
+        <v>45828</v>
+      </c>
+      <c r="D36" t="s">
+        <v>85</v>
+      </c>
+      <c r="E36" t="s">
+        <v>95</v>
+      </c>
+      <c r="F36" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>78</v>
+      </c>
+      <c r="B37" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="3">
+        <v>45829</v>
+      </c>
+      <c r="D37" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37" t="s">
+        <v>95</v>
+      </c>
+      <c r="F37" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" s="3">
+        <v>45829</v>
+      </c>
+      <c r="D38" t="s">
+        <v>85</v>
+      </c>
+      <c r="E38" t="s">
+        <v>95</v>
+      </c>
+      <c r="F38" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>80</v>
+      </c>
+      <c r="B39" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" s="3">
+        <v>45829</v>
+      </c>
+      <c r="D39" t="s">
+        <v>86</v>
+      </c>
+      <c r="E39" t="s">
+        <v>96</v>
+      </c>
+      <c r="F39" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 6.24.25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="139">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/20/2025, 6/21/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/20/2025, 6/21/2025)</t>
+    <t>Adoptions (06/23/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/23/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -113,30 +113,42 @@
     <t>2025-06-26</t>
   </si>
   <si>
-    <t>A0058734302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Cat Isolation 234, Cage 2</t>
+    <t>A0058763771</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Isolation 231, Cage 4</t>
+  </si>
+  <si>
+    <t>No Review Date</t>
+  </si>
+  <si>
+    <t>A0035002298</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ICU, 01 - B</t>
+  </si>
+  <si>
+    <t>A0058727432</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Multi Animal Holding</t>
   </si>
   <si>
     <t>2025-06-24</t>
   </si>
   <si>
-    <t>A0035002298</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 01 - B</t>
-  </si>
-  <si>
-    <t>No Review Date</t>
-  </si>
-  <si>
-    <t>A0058727432</t>
+    <t>A0058764920</t>
   </si>
   <si>
     <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 1</t>
   </si>
   <si>
+    <t>A0058765684</t>
+  </si>
+  <si>
+    <t>2025-06-30</t>
+  </si>
+  <si>
     <t>AnimalNumber</t>
   </si>
   <si>
@@ -155,220 +167,259 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058581988</t>
-  </si>
-  <si>
-    <t>A0058727921</t>
-  </si>
-  <si>
-    <t>A0058729123</t>
-  </si>
-  <si>
-    <t>A0058748113</t>
-  </si>
-  <si>
-    <t>A0058748530</t>
-  </si>
-  <si>
-    <t>A0058748533</t>
-  </si>
-  <si>
-    <t>A0058748536</t>
-  </si>
-  <si>
-    <t>A0058748541</t>
-  </si>
-  <si>
-    <t>A0058748559</t>
-  </si>
-  <si>
-    <t>A0058748561</t>
-  </si>
-  <si>
-    <t>A0058748566</t>
-  </si>
-  <si>
-    <t>A0058748569</t>
-  </si>
-  <si>
-    <t>A0058748790</t>
-  </si>
-  <si>
-    <t>A0058748794</t>
-  </si>
-  <si>
-    <t>A0058749076</t>
-  </si>
-  <si>
-    <t>A0058752173</t>
-  </si>
-  <si>
-    <t>A0058755847</t>
-  </si>
-  <si>
-    <t>A0058757630</t>
-  </si>
-  <si>
-    <t>A0058757640</t>
-  </si>
-  <si>
-    <t>A0058758488</t>
-  </si>
-  <si>
-    <t>A0058622436</t>
-  </si>
-  <si>
-    <t>A0058753935</t>
-  </si>
-  <si>
-    <t>A0058753940</t>
-  </si>
-  <si>
-    <t>A0058753950</t>
-  </si>
-  <si>
-    <t>A0058753956</t>
-  </si>
-  <si>
-    <t>A0058753958</t>
-  </si>
-  <si>
-    <t>A0058753963</t>
-  </si>
-  <si>
-    <t>A0058753970</t>
-  </si>
-  <si>
-    <t>A0058753979</t>
-  </si>
-  <si>
-    <t>A0058753987</t>
-  </si>
-  <si>
-    <t>A0058747360</t>
-  </si>
-  <si>
-    <t>A0058747362</t>
-  </si>
-  <si>
-    <t>A0058755856</t>
-  </si>
-  <si>
-    <t>A0058755861</t>
-  </si>
-  <si>
-    <t>A0058757250</t>
+    <t>A0058454216</t>
+  </si>
+  <si>
+    <t>A0058568926</t>
+  </si>
+  <si>
+    <t>A0058763197</t>
+  </si>
+  <si>
+    <t>A0016850435</t>
+  </si>
+  <si>
+    <t>A0047809430</t>
+  </si>
+  <si>
+    <t>A0051707058</t>
+  </si>
+  <si>
+    <t>A0057996204</t>
+  </si>
+  <si>
+    <t>A0057996215</t>
+  </si>
+  <si>
+    <t>A0057996233</t>
+  </si>
+  <si>
+    <t>A0057996245</t>
+  </si>
+  <si>
+    <t>A0058588779</t>
+  </si>
+  <si>
+    <t>A0058729684</t>
+  </si>
+  <si>
+    <t>A0058729698</t>
+  </si>
+  <si>
+    <t>A0058729703</t>
+  </si>
+  <si>
+    <t>A0058729706</t>
+  </si>
+  <si>
+    <t>A0058729710</t>
+  </si>
+  <si>
+    <t>A0058734134</t>
+  </si>
+  <si>
+    <t>A0058734140</t>
+  </si>
+  <si>
+    <t>A0058734147</t>
+  </si>
+  <si>
+    <t>A0058749349</t>
+  </si>
+  <si>
+    <t>A0058763044</t>
+  </si>
+  <si>
+    <t>A0058764550</t>
+  </si>
+  <si>
+    <t>A0058764565</t>
+  </si>
+  <si>
+    <t>A0058765306</t>
+  </si>
+  <si>
+    <t>A0058767718</t>
+  </si>
+  <si>
+    <t>A0058767736</t>
+  </si>
+  <si>
+    <t>A0058763999</t>
+  </si>
+  <si>
+    <t>A0058764006</t>
+  </si>
+  <si>
+    <t>A0058762583</t>
+  </si>
+  <si>
+    <t>A0058762584</t>
+  </si>
+  <si>
+    <t>A0058762585</t>
+  </si>
+  <si>
+    <t>A0058762586</t>
+  </si>
+  <si>
+    <t>A0058762960</t>
+  </si>
+  <si>
+    <t>A0058763173</t>
+  </si>
+  <si>
+    <t>A0058763174</t>
+  </si>
+  <si>
+    <t>A0058763177</t>
+  </si>
+  <si>
+    <t>A0058763180</t>
+  </si>
+  <si>
+    <t>A0058763319</t>
+  </si>
+  <si>
+    <t>A0058763584</t>
+  </si>
+  <si>
+    <t>A0058765957</t>
+  </si>
+  <si>
+    <t>A0058767738</t>
+  </si>
+  <si>
+    <t>A0058764479</t>
   </si>
   <si>
     <t>Rabbit</t>
   </si>
   <si>
+    <t>Rodent</t>
+  </si>
+  <si>
+    <t>Reptile/Amphibian</t>
+  </si>
+  <si>
+    <t>Clinic</t>
+  </si>
+  <si>
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
+    <t>Seized / Custody</t>
+  </si>
+  <si>
+    <t>Stray</t>
+  </si>
+  <si>
+    <t>Transfer In</t>
+  </si>
+  <si>
+    <t>Retention</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Guardian Surrender - FIELD!</t>
+  </si>
+  <si>
+    <t>Evaluation/Poss Adopt - OTC!</t>
+  </si>
+  <si>
+    <t>Euthanasia Request - OTC!</t>
+  </si>
+  <si>
+    <t>Guardian Surrender - OTC!</t>
+  </si>
+  <si>
+    <t>Evaluation/Poss Adopt - FIELD!</t>
+  </si>
+  <si>
+    <t>DOA</t>
+  </si>
+  <si>
+    <t>Signed Over</t>
+  </si>
+  <si>
+    <t>OTC</t>
+  </si>
+  <si>
+    <t>Born in Care</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>Abandoned by owner - OTC!</t>
+  </si>
+  <si>
+    <t>ACO or DCO in County</t>
+  </si>
+  <si>
+    <t>Clinic - Retention</t>
+  </si>
+  <si>
+    <t>Clinic - Stray</t>
+  </si>
+  <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Seized – General</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
+    <t>Seized – Eviction</t>
+  </si>
+  <si>
+    <t>Seized – Police</t>
+  </si>
+  <si>
+    <t>Seized – Owner Died</t>
+  </si>
+  <si>
+    <t>Seized – Order Violation</t>
+  </si>
+  <si>
+    <t>Seized - Hoarding</t>
+  </si>
+  <si>
     <t>Return</t>
   </si>
   <si>
-    <t>Seized / Custody</t>
-  </si>
-  <si>
-    <t>Stray</t>
-  </si>
-  <si>
-    <t>Transfer In</t>
-  </si>
-  <si>
-    <t>Evaluation/Poss Adopt - OTC!</t>
-  </si>
-  <si>
-    <t>Euthanasia Request - OTC!</t>
-  </si>
-  <si>
-    <t>Evaluation/Poss Adopt - FIELD!</t>
-  </si>
-  <si>
-    <t>OTC</t>
-  </si>
-  <si>
-    <t>Euthanasia Request - FIELD!</t>
-  </si>
-  <si>
-    <t>Guardian Surrender - FIELD!</t>
-  </si>
-  <si>
-    <t>Owned 30 Days or Less - OTC!</t>
-  </si>
-  <si>
-    <t>Signed Over</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>Vet clinic</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
-  </si>
-  <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
-    <t>Seized – General</t>
-  </si>
-  <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
-    <t>Seized – Eviction</t>
-  </si>
-  <si>
-    <t>Seized – Police</t>
-  </si>
-  <si>
-    <t>Seized – Owner Died</t>
-  </si>
-  <si>
-    <t>Seized – Order Violation</t>
-  </si>
-  <si>
-    <t>Seized - Hoarding</t>
-  </si>
-  <si>
     <t>OTC - OS - SAFE</t>
   </si>
   <si>
     <t>Clinic - Medical Treatment</t>
-  </si>
-  <si>
-    <t>Clinic - Stray</t>
-  </si>
-  <si>
-    <t>Clinic - Retention</t>
   </si>
   <si>
     <t>Clinic - Case Assistance</t>
@@ -757,7 +808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -777,7 +828,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -785,7 +836,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -801,7 +852,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -809,7 +860,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -817,7 +868,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -841,7 +892,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -857,7 +908,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>18</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -865,7 +916,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -889,7 +940,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -908,7 +959,7 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="C20">
         <v>27</v>
@@ -919,10 +970,10 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C21">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -930,10 +981,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="C22">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -944,7 +995,7 @@
         <v>30</v>
       </c>
       <c r="C23">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -952,7 +1003,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -963,10 +1014,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>133</v>
+        <v>161</v>
       </c>
       <c r="C25">
-        <v>219</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1010,206 +1061,228 @@
         <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" t="s">
         <v>38</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>39</v>
       </c>
-      <c r="C31" t="s">
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C34" s="1" t="s">
+    <row r="33" spans="1:4">
+      <c r="A33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
-        <v>86</v>
-      </c>
-      <c r="B35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C37">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>100</v>
-      </c>
-      <c r="C38">
+        <v>107</v>
+      </c>
+      <c r="D38">
         <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>104</v>
+        <v>118</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
+      </c>
+      <c r="D39">
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>99</v>
-      </c>
-      <c r="B40">
-        <v>3</v>
-      </c>
-      <c r="C40">
-        <v>8</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>106</v>
+        <v>116</v>
+      </c>
+      <c r="B42">
+        <v>9</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>101</v>
-      </c>
-      <c r="B45">
-        <v>6</v>
-      </c>
-      <c r="C45">
-        <v>3</v>
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>110</v>
+        <v>119</v>
+      </c>
+      <c r="B47">
+        <v>2</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>83</v>
-      </c>
-      <c r="C51">
-        <v>1</v>
+        <v>130</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>85</v>
-      </c>
-      <c r="B52">
-        <v>6</v>
-      </c>
-      <c r="D52">
-        <v>1</v>
+        <v>131</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>97</v>
-      </c>
-      <c r="B53">
-        <v>1</v>
-      </c>
-      <c r="C53">
-        <v>1</v>
-      </c>
-      <c r="D53">
-        <v>2</v>
+        <v>132</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>114</v>
+        <v>98</v>
+      </c>
+      <c r="B54">
+        <v>14</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>115</v>
+        <v>117</v>
+      </c>
+      <c r="B55">
+        <v>7</v>
+      </c>
+      <c r="C55">
+        <v>3</v>
+      </c>
+      <c r="D55">
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>118</v>
+        <v>115</v>
+      </c>
+      <c r="B58">
+        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>114</v>
+      </c>
+      <c r="D59">
+        <v>2</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>120</v>
+        <v>135</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>121</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1219,787 +1292,927 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="C2" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="E2" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="F2" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="C3" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D3" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="E3" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="F3" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D4" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="E4" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="F4" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D5" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E5" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="F5" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D6" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E6" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="F6" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
         <v>21</v>
       </c>
       <c r="C7" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D7" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E7" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="F7" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D8" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E8" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="F8" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D9" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E9" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="F9" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D10" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E10" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="F10" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D11" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E11" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="F11" t="s">
-        <v>99</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>92</v>
       </c>
       <c r="C12" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D12" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>89</v>
+        <v>104</v>
       </c>
       <c r="F12" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D13" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E13" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D14" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E14" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="F14" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D15" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E15" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="F15" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D16" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E16" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="F16" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C17" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D17" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E17" t="s">
-        <v>90</v>
+        <v>105</v>
       </c>
       <c r="F17" t="s">
-        <v>97</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D18" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E18" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="F18" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="C19" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D19" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E19" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="F19" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B20" t="s">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="C20" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D20" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E20" t="s">
-        <v>87</v>
+        <v>106</v>
       </c>
       <c r="F20" t="s">
-        <v>97</v>
+        <v>116</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="C21" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D21" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="E21" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="F21" t="s">
-        <v>99</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
         <v>21</v>
       </c>
       <c r="C22" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D22" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="E22" t="s">
-        <v>93</v>
+        <v>104</v>
       </c>
       <c r="F22" t="s">
-        <v>83</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C23" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D23" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E23" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="F23" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B24" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C24" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D24" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E24" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="F24" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>40</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="C25" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D25" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E25" t="s">
-        <v>94</v>
+        <v>105</v>
       </c>
       <c r="F25" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>93</v>
       </c>
       <c r="C26" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D26" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E26" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="F26" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B27" t="s">
         <v>20</v>
       </c>
       <c r="C27" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D27" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E27" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F27" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B28" t="s">
         <v>20</v>
       </c>
       <c r="C28" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D28" t="s">
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="E28" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F28" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B29" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C29" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D29" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="E29" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="F29" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C30" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D30" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="E30" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="F30" t="s">
-        <v>101</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B31" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C31" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D31" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="E31" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="F31" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="B32" t="s">
         <v>20</v>
       </c>
       <c r="C32" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D32" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="E32" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="F32" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="B33" t="s">
         <v>20</v>
       </c>
       <c r="C33" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D33" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="E33" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="F33" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="B34" t="s">
-        <v>81</v>
+        <v>20</v>
       </c>
       <c r="C34" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D34" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="E34" t="s">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="F34" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B35" t="s">
         <v>20</v>
       </c>
       <c r="C35" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D35" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="E35" t="s">
-        <v>95</v>
+        <v>110</v>
       </c>
       <c r="F35" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="B36" t="s">
         <v>20</v>
       </c>
       <c r="C36" s="3">
-        <v>45828</v>
+        <v>45831</v>
       </c>
       <c r="D36" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="E36" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F36" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="B37" t="s">
         <v>20</v>
       </c>
       <c r="C37" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D37" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="E37" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F37" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B38" t="s">
         <v>20</v>
       </c>
       <c r="C38" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D38" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="E38" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="F38" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="B39" t="s">
         <v>20</v>
       </c>
       <c r="C39" s="3">
-        <v>45829</v>
+        <v>45831</v>
       </c>
       <c r="D39" t="s">
-        <v>86</v>
+        <v>98</v>
       </c>
       <c r="E39" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
       <c r="F39" t="s">
-        <v>86</v>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
+        <v>87</v>
+      </c>
+      <c r="B40" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D40" t="s">
+        <v>98</v>
+      </c>
+      <c r="E40" t="s">
+        <v>112</v>
+      </c>
+      <c r="F40" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>88</v>
+      </c>
+      <c r="B41" t="s">
+        <v>20</v>
+      </c>
+      <c r="C41" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D41" t="s">
+        <v>98</v>
+      </c>
+      <c r="E41" t="s">
+        <v>109</v>
+      </c>
+      <c r="F41" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" t="s">
+        <v>32</v>
+      </c>
+      <c r="B42" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D42" t="s">
+        <v>98</v>
+      </c>
+      <c r="E42" t="s">
+        <v>109</v>
+      </c>
+      <c r="F42" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" t="s">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>94</v>
+      </c>
+      <c r="C43" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D43" t="s">
+        <v>98</v>
+      </c>
+      <c r="E43" t="s">
+        <v>109</v>
+      </c>
+      <c r="F43" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" t="s">
+        <v>89</v>
+      </c>
+      <c r="B44" t="s">
+        <v>20</v>
+      </c>
+      <c r="C44" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D44" t="s">
+        <v>98</v>
+      </c>
+      <c r="E44" t="s">
+        <v>111</v>
+      </c>
+      <c r="F44" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" t="s">
+        <v>90</v>
+      </c>
+      <c r="B45" t="s">
+        <v>20</v>
+      </c>
+      <c r="C45" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D45" t="s">
+        <v>98</v>
+      </c>
+      <c r="E45" t="s">
+        <v>111</v>
+      </c>
+      <c r="F45" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" s="3">
+        <v>45831</v>
+      </c>
+      <c r="D46" t="s">
+        <v>99</v>
+      </c>
+      <c r="E46" t="s">
+        <v>113</v>
+      </c>
+      <c r="F46" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated data for 6/26/25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="86">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/24/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/24/2025)</t>
+    <t>Adoptions (06/25/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/25/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -128,13 +128,7 @@
     <t xml:space="preserve">  ICU, 01 - B</t>
   </si>
   <si>
-    <t>No Review Date</t>
-  </si>
-  <si>
-    <t>A0058764920</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 1</t>
+    <t>2025-06-26</t>
   </si>
   <si>
     <t>A0058765684</t>
@@ -164,136 +158,97 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058589089</t>
-  </si>
-  <si>
-    <t>A0058718599</t>
-  </si>
-  <si>
-    <t>A0058734634</t>
-  </si>
-  <si>
-    <t>A0058770794</t>
-  </si>
-  <si>
-    <t>A0058772641</t>
-  </si>
-  <si>
-    <t>A0058772686</t>
-  </si>
-  <si>
-    <t>A0058772993</t>
-  </si>
-  <si>
-    <t>A0058775218</t>
-  </si>
-  <si>
-    <t>A0053747735</t>
-  </si>
-  <si>
-    <t>A0058774353</t>
-  </si>
-  <si>
-    <t>A0058770859</t>
-  </si>
-  <si>
-    <t>A0058773648</t>
-  </si>
-  <si>
-    <t>A0058770648</t>
-  </si>
-  <si>
-    <t>Rabbit</t>
-  </si>
-  <si>
-    <t>Rodent</t>
+    <t>A0058779670</t>
+  </si>
+  <si>
+    <t>A0058780889</t>
+  </si>
+  <si>
+    <t>A0058783844</t>
+  </si>
+  <si>
+    <t>A0058780905</t>
+  </si>
+  <si>
+    <t>A0058781169</t>
   </si>
   <si>
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
+    <t>Seized / Custody</t>
+  </si>
+  <si>
+    <t>Stray</t>
+  </si>
+  <si>
+    <t>Euthanasia Request - OTC!</t>
+  </si>
+  <si>
+    <t>DOA</t>
+  </si>
+  <si>
+    <t>Guardian Surrender - OTC!</t>
+  </si>
+  <si>
+    <t>Signed Over</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
+    <t>Transfer In</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Seized – General</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
+    <t>Seized – Eviction</t>
+  </si>
+  <si>
+    <t>Seized – Police</t>
+  </si>
+  <si>
+    <t>Seized – Owner Died</t>
+  </si>
+  <si>
+    <t>Seized – Order Violation</t>
+  </si>
+  <si>
+    <t>Seized - Hoarding</t>
+  </si>
+  <si>
     <t>Return</t>
-  </si>
-  <si>
-    <t>Seized / Custody</t>
-  </si>
-  <si>
-    <t>Stray</t>
-  </si>
-  <si>
-    <t>Transfer In</t>
-  </si>
-  <si>
-    <t>Euthanasia Request - OTC!</t>
-  </si>
-  <si>
-    <t>Evaluation/Poss Adopt - OTC!</t>
-  </si>
-  <si>
-    <t>OTC</t>
-  </si>
-  <si>
-    <t>Owned More than 30 Days - OTC!</t>
-  </si>
-  <si>
-    <t>Signed Over</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>ACO or DCO in County</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
-  </si>
-  <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
-    <t>Seized – General</t>
-  </si>
-  <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
-    <t>Seized – Eviction</t>
-  </si>
-  <si>
-    <t>Seized – Police</t>
-  </si>
-  <si>
-    <t>Seized – Owner Died</t>
-  </si>
-  <si>
-    <t>Seized – Order Violation</t>
-  </si>
-  <si>
-    <t>Seized - Hoarding</t>
   </si>
   <si>
     <t>OTC - OS - SAFE</t>
@@ -694,7 +649,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -714,7 +669,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>5</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -722,7 +677,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -738,7 +693,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -778,7 +733,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -794,7 +749,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -802,7 +757,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>19</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -826,7 +781,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -845,10 +800,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="C20">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -856,10 +811,10 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="C21">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -867,10 +822,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="C22">
-        <v>135</v>
+        <v>141</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -900,10 +855,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>168</v>
+        <v>141</v>
       </c>
       <c r="C25">
-        <v>202</v>
+        <v>211</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -958,191 +913,171 @@
         <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" t="s">
         <v>40</v>
       </c>
-      <c r="B32" t="s">
-        <v>41</v>
-      </c>
-      <c r="C32" t="s">
-        <v>42</v>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="35" spans="1:4">
-      <c r="A35" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>23</v>
+      <c r="A35" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>68</v>
-      </c>
-      <c r="C36">
+        <v>56</v>
+      </c>
+      <c r="B36">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>60</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>76</v>
-      </c>
-      <c r="C38">
-        <v>3</v>
-      </c>
-      <c r="D38">
-        <v>1</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>87</v>
+        <v>62</v>
+      </c>
+      <c r="B45">
+        <v>1</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>78</v>
-      </c>
-      <c r="C46">
-        <v>1</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>67</v>
-      </c>
-      <c r="B53">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4">
+        <v>61</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>77</v>
-      </c>
-      <c r="B54">
-        <v>3</v>
-      </c>
-      <c r="D54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="A62" t="s">
-        <v>100</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -1152,307 +1087,127 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>21</v>
       </c>
       <c r="C2" s="3">
-        <v>45832</v>
+        <v>45833</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="E2" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3">
-        <v>45832</v>
+        <v>45833</v>
       </c>
       <c r="D3" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>76</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="C4" s="3">
-        <v>45832</v>
+        <v>45833</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="F4" t="s">
-        <v>77</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45832</v>
+        <v>45833</v>
       </c>
       <c r="D5" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="F5" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45832</v>
+        <v>45833</v>
       </c>
       <c r="D6" t="s">
-        <v>64</v>
+        <v>54</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="F6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
         <v>54</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D7" t="s">
-        <v>64</v>
-      </c>
-      <c r="E7" t="s">
-        <v>70</v>
-      </c>
-      <c r="F7" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D8" t="s">
-        <v>64</v>
-      </c>
-      <c r="E8" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D9" t="s">
-        <v>64</v>
-      </c>
-      <c r="E9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>57</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D10" t="s">
-        <v>65</v>
-      </c>
-      <c r="E10" t="s">
-        <v>72</v>
-      </c>
-      <c r="F10" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>58</v>
-      </c>
-      <c r="B11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D11" t="s">
-        <v>66</v>
-      </c>
-      <c r="E11" t="s">
-        <v>73</v>
-      </c>
-      <c r="F11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D12" t="s">
-        <v>67</v>
-      </c>
-      <c r="E12" t="s">
-        <v>71</v>
-      </c>
-      <c r="F12" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>59</v>
-      </c>
-      <c r="B13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D13" t="s">
-        <v>67</v>
-      </c>
-      <c r="E13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D14" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" t="s">
-        <v>71</v>
-      </c>
-      <c r="F14" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" t="s">
-        <v>61</v>
-      </c>
-      <c r="B15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="3">
-        <v>45832</v>
-      </c>
-      <c r="D15" t="s">
-        <v>68</v>
-      </c>
-      <c r="E15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F15" t="s">
-        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 6.27.25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="117">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/25/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/25/2025)</t>
+    <t>Adoptions (06/26/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/26/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -113,22 +113,19 @@
     <t>2025-06-28</t>
   </si>
   <si>
-    <t>A0058763771</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Cat Isolation 231, Cage 4</t>
-  </si>
-  <si>
-    <t>2025-06-27</t>
-  </si>
-  <si>
-    <t>A0035002298</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 01 - B</t>
-  </si>
-  <si>
-    <t>2025-06-26</t>
+    <t>A0058789119</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Treatment, B</t>
+  </si>
+  <si>
+    <t>2025-07-01</t>
+  </si>
+  <si>
+    <t>A0058795880</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ICU, 02</t>
   </si>
   <si>
     <t>A0058765684</t>
@@ -158,60 +155,168 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058779670</t>
-  </si>
-  <si>
-    <t>A0058780889</t>
-  </si>
-  <si>
-    <t>A0058783844</t>
-  </si>
-  <si>
-    <t>A0058780905</t>
-  </si>
-  <si>
-    <t>A0058781169</t>
+    <t>A0057606321</t>
+  </si>
+  <si>
+    <t>A0057606331</t>
+  </si>
+  <si>
+    <t>A0057606333</t>
+  </si>
+  <si>
+    <t>A0058647055</t>
+  </si>
+  <si>
+    <t>A0058757250</t>
+  </si>
+  <si>
+    <t>A0058771476</t>
+  </si>
+  <si>
+    <t>A0058779323</t>
+  </si>
+  <si>
+    <t>A0058787827</t>
+  </si>
+  <si>
+    <t>A0058789307</t>
+  </si>
+  <si>
+    <t>A0058344428</t>
+  </si>
+  <si>
+    <t>A0058703414</t>
+  </si>
+  <si>
+    <t>A0058718252</t>
+  </si>
+  <si>
+    <t>A0058787487</t>
+  </si>
+  <si>
+    <t>A0058787489</t>
+  </si>
+  <si>
+    <t>A0058787491</t>
+  </si>
+  <si>
+    <t>A0058787494</t>
+  </si>
+  <si>
+    <t>A0058787496</t>
+  </si>
+  <si>
+    <t>A0058787499</t>
+  </si>
+  <si>
+    <t>A0058787532</t>
+  </si>
+  <si>
+    <t>A0058792719</t>
+  </si>
+  <si>
+    <t>A0058792732</t>
+  </si>
+  <si>
+    <t>A0058778873</t>
+  </si>
+  <si>
+    <t>A0058787259</t>
+  </si>
+  <si>
+    <t>A0058787263</t>
+  </si>
+  <si>
+    <t>A0058787609</t>
+  </si>
+  <si>
+    <t>A0058790016</t>
+  </si>
+  <si>
+    <t>A0058793704</t>
+  </si>
+  <si>
+    <t>A0058793726</t>
+  </si>
+  <si>
+    <t>A0058793733</t>
+  </si>
+  <si>
+    <t>Rabbit</t>
+  </si>
+  <si>
+    <t>Clinic</t>
   </si>
   <si>
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
+    <t>Return</t>
+  </si>
+  <si>
     <t>Seized / Custody</t>
   </si>
   <si>
     <t>Stray</t>
   </si>
   <si>
+    <t>Case - Outreach</t>
+  </si>
+  <si>
     <t>Euthanasia Request - OTC!</t>
   </si>
   <si>
+    <t>Evaluation/Poss Adopt - OTC!</t>
+  </si>
+  <si>
+    <t>Owned 30 Days or Less - OTC!</t>
+  </si>
+  <si>
+    <t>Signed Over</t>
+  </si>
+  <si>
+    <t>Eviction</t>
+  </si>
+  <si>
+    <t>Cruelty</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>OTC</t>
+  </si>
+  <si>
+    <t>Abandoned by owner - OTC!</t>
+  </si>
+  <si>
+    <t>Clinic - Case Assistance - Outreach</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Seized – Eviction</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
+    <t>Transfer In</t>
+  </si>
+  <si>
     <t>DOA</t>
   </si>
   <si>
-    <t>Guardian Surrender - OTC!</t>
-  </si>
-  <si>
-    <t>Signed Over</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Transfer In</t>
-  </si>
-  <si>
     <t>Euthanasia Req – Field</t>
   </si>
   <si>
@@ -224,18 +329,12 @@
     <t>Seized – Abandoned</t>
   </si>
   <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
     <t>Seized – General</t>
   </si>
   <si>
     <t>Seized – Hospital</t>
   </si>
   <si>
-    <t>Seized – Eviction</t>
-  </si>
-  <si>
     <t>Seized – Police</t>
   </si>
   <si>
@@ -248,9 +347,6 @@
     <t>Seized - Hoarding</t>
   </si>
   <si>
-    <t>Return</t>
-  </si>
-  <si>
     <t>OTC - OS - SAFE</t>
   </si>
   <si>
@@ -264,9 +360,6 @@
   </si>
   <si>
     <t>Clinic - Case Assistance</t>
-  </si>
-  <si>
-    <t>Clinic - Case Assistance - Outreach</t>
   </si>
   <si>
     <t>Clinic - Outreach</t>
@@ -669,7 +762,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>21</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -677,7 +770,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -693,7 +786,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>199</v>
+        <v>190</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -709,7 +802,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -733,7 +826,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>20</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -741,7 +834,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -749,7 +842,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -757,7 +850,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -765,7 +858,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -781,7 +874,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -800,10 +893,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C20">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -811,10 +904,10 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C21">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -822,10 +915,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="C22">
-        <v>141</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -833,7 +926,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C23">
         <v>22</v>
@@ -844,7 +937,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -855,10 +948,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>141</v>
+        <v>168</v>
       </c>
       <c r="C25">
-        <v>211</v>
+        <v>199</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -902,23 +995,23 @@
         <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
+        <v>37</v>
+      </c>
+      <c r="B31" t="s">
         <v>38</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>39</v>
-      </c>
-      <c r="C31" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="1" t="s">
-        <v>63</v>
+        <v>97</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>20</v>
@@ -932,20 +1025,20 @@
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>56</v>
-      </c>
-      <c r="B36">
-        <v>1</v>
+        <v>99</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>60</v>
+        <v>92</v>
+      </c>
+      <c r="B37">
+        <v>3</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -953,131 +1046,152 @@
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>65</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>66</v>
+        <v>101</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>67</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>69</v>
+        <v>96</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>70</v>
+        <v>104</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="B45">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>72</v>
+        <v>95</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
+        <v>78</v>
+      </c>
+      <c r="B51">
+        <v>2</v>
+      </c>
+      <c r="C51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>80</v>
       </c>
       <c r="B52">
+        <v>7</v>
+      </c>
+      <c r="D52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" t="s">
+        <v>93</v>
+      </c>
+      <c r="B53">
         <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
-        <v>61</v>
       </c>
       <c r="C53">
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3">
+        <v>91</v>
+      </c>
+      <c r="B59">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
       <c r="A61" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1087,127 +1201,627 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="E2" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="F2" t="s">
-        <v>60</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
       </c>
       <c r="C3" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
-        <v>56</v>
+        <v>81</v>
       </c>
       <c r="F3" t="s">
-        <v>56</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="E4" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="F4" t="s">
-        <v>61</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="3">
-        <v>45833</v>
+        <v>45834</v>
       </c>
       <c r="D5" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="F5" t="s">
-        <v>62</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E6" t="s">
+        <v>83</v>
+      </c>
+      <c r="F6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
         <v>51</v>
       </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="3">
-        <v>45833</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D7" t="s">
+        <v>77</v>
+      </c>
+      <c r="E7" t="s">
+        <v>82</v>
+      </c>
+      <c r="F7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D8" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D9" t="s">
+        <v>77</v>
+      </c>
+      <c r="E9" t="s">
+        <v>83</v>
+      </c>
+      <c r="F9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
         <v>54</v>
       </c>
-      <c r="E6" t="s">
+      <c r="B10" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" t="s">
+        <v>82</v>
+      </c>
+      <c r="F10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D11" t="s">
+        <v>78</v>
+      </c>
+      <c r="E11" t="s">
+        <v>82</v>
+      </c>
+      <c r="F11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D12" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D13" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" t="s">
+        <v>84</v>
+      </c>
+      <c r="F13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D14" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" t="s">
+        <v>85</v>
+      </c>
+      <c r="F14" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
         <v>59</v>
       </c>
-      <c r="F6" t="s">
-        <v>54</v>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B16" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D16" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" t="s">
+        <v>85</v>
+      </c>
+      <c r="F16" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D17" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D18" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" t="s">
+        <v>85</v>
+      </c>
+      <c r="F18" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D19" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" t="s">
+        <v>85</v>
+      </c>
+      <c r="F19" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D20" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" t="s">
+        <v>86</v>
+      </c>
+      <c r="F20" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E21" t="s">
+        <v>87</v>
+      </c>
+      <c r="F21" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D22" t="s">
+        <v>79</v>
+      </c>
+      <c r="E22" t="s">
+        <v>87</v>
+      </c>
+      <c r="F22" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>67</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E23" t="s">
+        <v>88</v>
+      </c>
+      <c r="F23" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>68</v>
+      </c>
+      <c r="B24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C24" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D24" t="s">
+        <v>80</v>
+      </c>
+      <c r="E24" t="s">
+        <v>89</v>
+      </c>
+      <c r="F24" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" t="s">
+        <v>75</v>
+      </c>
+      <c r="C25" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D25" t="s">
+        <v>80</v>
+      </c>
+      <c r="E25" t="s">
+        <v>89</v>
+      </c>
+      <c r="F25" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D26" t="s">
+        <v>80</v>
+      </c>
+      <c r="E26" t="s">
+        <v>88</v>
+      </c>
+      <c r="F26" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D27" t="s">
+        <v>80</v>
+      </c>
+      <c r="E27" t="s">
+        <v>89</v>
+      </c>
+      <c r="F27" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D28" t="s">
+        <v>80</v>
+      </c>
+      <c r="E28" t="s">
+        <v>88</v>
+      </c>
+      <c r="F28" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D29" t="s">
+        <v>80</v>
+      </c>
+      <c r="E29" t="s">
+        <v>90</v>
+      </c>
+      <c r="F29" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D30" t="s">
+        <v>80</v>
+      </c>
+      <c r="E30" t="s">
+        <v>88</v>
+      </c>
+      <c r="F30" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>74</v>
+      </c>
+      <c r="B31" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="3">
+        <v>45834</v>
+      </c>
+      <c r="D31" t="s">
+        <v>80</v>
+      </c>
+      <c r="E31" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 7.1.25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="111">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/27/2025, 06/28/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/27/2025, 06/28/2025)</t>
+    <t>Adoptions (06/30/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (06/30/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -113,19 +113,22 @@
     <t>2025-07-02</t>
   </si>
   <si>
-    <t>A0058795880</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 02</t>
-  </si>
-  <si>
-    <t>2025-07-01</t>
-  </si>
-  <si>
-    <t>A0058796476</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 03 - A</t>
+    <t>A0058812302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  ICU, 01</t>
+  </si>
+  <si>
+    <t>2025-07-05</t>
+  </si>
+  <si>
+    <t>A0058812861</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 2</t>
+  </si>
+  <si>
+    <t>2025-07-07</t>
   </si>
   <si>
     <t>AnimalNumber</t>
@@ -146,138 +149,84 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058805230</t>
+    <t>A0058563467</t>
+  </si>
+  <si>
+    <t>A0058772179</t>
+  </si>
+  <si>
+    <t>A0058816447</t>
+  </si>
+  <si>
+    <t>A0015599570</t>
   </si>
   <si>
     <t>A0054021734</t>
   </si>
   <si>
-    <t>A0058780847</t>
-  </si>
-  <si>
-    <t>A0058787214</t>
-  </si>
-  <si>
-    <t>A0058790320</t>
-  </si>
-  <si>
-    <t>A0058800447</t>
-  </si>
-  <si>
-    <t>A0058800763</t>
-  </si>
-  <si>
-    <t>A0058803369</t>
-  </si>
-  <si>
-    <t>A0058804124</t>
-  </si>
-  <si>
-    <t>A0058804353</t>
-  </si>
-  <si>
-    <t>A0058805787</t>
-  </si>
-  <si>
-    <t>A0058805800</t>
-  </si>
-  <si>
-    <t>A0058805811</t>
-  </si>
-  <si>
-    <t>A0058373583</t>
-  </si>
-  <si>
-    <t>A0058640973</t>
-  </si>
-  <si>
-    <t>A0058797987</t>
-  </si>
-  <si>
-    <t>A0058798000</t>
-  </si>
-  <si>
-    <t>A0058798054</t>
-  </si>
-  <si>
-    <t>A0058801947</t>
-  </si>
-  <si>
-    <t>A0058801964</t>
-  </si>
-  <si>
-    <t>A0058806595</t>
-  </si>
-  <si>
-    <t>A0040017266</t>
-  </si>
-  <si>
-    <t>A0058790535</t>
-  </si>
-  <si>
-    <t>A0058790545</t>
-  </si>
-  <si>
-    <t>A0058790552</t>
-  </si>
-  <si>
-    <t>A0058790558</t>
-  </si>
-  <si>
-    <t>A0058790560</t>
-  </si>
-  <si>
-    <t>A0058795591</t>
-  </si>
-  <si>
-    <t>A0058796649</t>
-  </si>
-  <si>
-    <t>A0058796651</t>
-  </si>
-  <si>
-    <t>A0058796654</t>
-  </si>
-  <si>
-    <t>A0058796655</t>
-  </si>
-  <si>
-    <t>A0058796658</t>
-  </si>
-  <si>
-    <t>A0058796660</t>
-  </si>
-  <si>
-    <t>A0058796661</t>
-  </si>
-  <si>
-    <t>A0058796664</t>
-  </si>
-  <si>
-    <t>A0058796665</t>
-  </si>
-  <si>
-    <t>A0058797788</t>
-  </si>
-  <si>
-    <t>A0058797907</t>
-  </si>
-  <si>
-    <t>A0058799429</t>
-  </si>
-  <si>
-    <t>A0058799431</t>
-  </si>
-  <si>
-    <t>Mammal</t>
-  </si>
-  <si>
-    <t>Reptile/Amphibian</t>
+    <t>A0058804211</t>
+  </si>
+  <si>
+    <t>A0058811219</t>
+  </si>
+  <si>
+    <t>A0058812472</t>
+  </si>
+  <si>
+    <t>A0058812728</t>
+  </si>
+  <si>
+    <t>A0058813263</t>
+  </si>
+  <si>
+    <t>A0058813495</t>
+  </si>
+  <si>
+    <t>A0058817552</t>
+  </si>
+  <si>
+    <t>A0058501223</t>
+  </si>
+  <si>
+    <t>A0058814043</t>
+  </si>
+  <si>
+    <t>A0058814049</t>
+  </si>
+  <si>
+    <t>A0058814052</t>
+  </si>
+  <si>
+    <t>A0058814056</t>
+  </si>
+  <si>
+    <t>A0058814060</t>
+  </si>
+  <si>
+    <t>A0058817102</t>
+  </si>
+  <si>
+    <t>A0058811036</t>
+  </si>
+  <si>
+    <t>A0058816089</t>
+  </si>
+  <si>
+    <t>A0058811183</t>
+  </si>
+  <si>
+    <t>A0058811207</t>
   </si>
   <si>
     <t>Rabbit</t>
   </si>
   <si>
+    <t>Domestic (Cage) Bird</t>
+  </si>
+  <si>
+    <t>Farm Type Fowl</t>
+  </si>
+  <si>
     <t>Clinic</t>
   </si>
   <si>
@@ -293,16 +242,28 @@
     <t>Stray</t>
   </si>
   <si>
+    <t>Transfer In</t>
+  </si>
+  <si>
+    <t>Retention</t>
+  </si>
+  <si>
     <t>Euthanasia Request - OTC!</t>
   </si>
   <si>
-    <t>Evaluation/Poss Adopt - OTC!</t>
-  </si>
-  <si>
-    <t>Owned 30 Days or Less - OTC!</t>
-  </si>
-  <si>
-    <t>Abandoned</t>
+    <t>DOA</t>
+  </si>
+  <si>
+    <t>Guardian Surrender - OTC!</t>
+  </si>
+  <si>
+    <t>OTC</t>
+  </si>
+  <si>
+    <t>Guardian Surrender - FIELD!</t>
+  </si>
+  <si>
+    <t>Owned More than 30 Days FIELD!</t>
   </si>
   <si>
     <t>Signed Over</t>
@@ -311,10 +272,13 @@
     <t>Owner died</t>
   </si>
   <si>
-    <t>OTC</t>
-  </si>
-  <si>
-    <t>No Hold</t>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>ACO or DCO in County</t>
+  </si>
+  <si>
+    <t>Clinic - Retention</t>
   </si>
   <si>
     <t>Clinic - Stray</t>
@@ -326,33 +290,27 @@
     <t>OTC – OS</t>
   </si>
   <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Seized – Owner Died</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
     <t>Seized – Abandoned</t>
   </si>
   <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Seized – Owner Died</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Transfer In</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
     <t>Seized – Cruelty</t>
   </si>
   <si>
@@ -378,9 +336,6 @@
   </si>
   <si>
     <t>Clinic - Medical Treatment</t>
-  </si>
-  <si>
-    <t>Clinic - Retention</t>
   </si>
   <si>
     <t>Clinic - Case Assistance</t>
@@ -789,7 +744,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>18</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -797,7 +752,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -813,7 +768,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -821,7 +776,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -829,7 +784,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -853,7 +808,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -861,7 +816,7 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -869,7 +824,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -877,7 +832,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -931,7 +886,7 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C21">
         <v>21</v>
@@ -942,10 +897,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C22">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -956,7 +911,7 @@
         <v>37</v>
       </c>
       <c r="C23">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -975,10 +930,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C25">
-        <v>208</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -1022,12 +977,12 @@
         <v>36</v>
       </c>
       <c r="C30" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1" t="s">
-        <v>106</v>
+        <v>95</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>20</v>
@@ -1041,87 +996,96 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>107</v>
+        <v>75</v>
+      </c>
+      <c r="C34">
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>108</v>
+        <v>78</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35">
+        <v>2</v>
+      </c>
+      <c r="D35">
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="B36">
-        <v>5</v>
-      </c>
-      <c r="C36">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>110</v>
+        <v>94</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>111</v>
+        <v>91</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>103</v>
-      </c>
-      <c r="B40">
-        <v>1</v>
-      </c>
-      <c r="C40">
-        <v>2</v>
+        <v>97</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>104</v>
-      </c>
-      <c r="B44">
-        <v>2</v>
+        <v>92</v>
+      </c>
+      <c r="D44">
+        <v>5</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="B47">
         <v>1</v>
@@ -1129,20 +1093,17 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>89</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1150,42 +1111,39 @@
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="B51">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="D51">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="B52">
         <v>1</v>
       </c>
       <c r="C52">
-        <v>2</v>
-      </c>
-      <c r="D52">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="B55">
         <v>1</v>
@@ -1193,27 +1151,30 @@
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>121</v>
+        <v>87</v>
+      </c>
+      <c r="D56">
+        <v>2</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>123</v>
+        <v>108</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>125</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -1223,907 +1184,527 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="C2" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F2" t="s">
         <v>87</v>
-      </c>
-      <c r="E2" t="s">
-        <v>91</v>
-      </c>
-      <c r="F2" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="C3" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D3" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="F3" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D4" t="s">
+        <v>70</v>
+      </c>
+      <c r="E4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" t="s">
         <v>88</v>
-      </c>
-      <c r="E4" t="s">
-        <v>92</v>
-      </c>
-      <c r="F4" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D5" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="F5" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D6" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E6" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="F6" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>68</v>
       </c>
       <c r="C7" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D7" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D8" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D9" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E9" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="F9" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D10" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E10" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="F10" t="s">
-        <v>101</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
         <v>21</v>
       </c>
       <c r="C11" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D11" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E11" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="F11" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="C12" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D12" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E12" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="F12" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D13" t="s">
-        <v>88</v>
+        <v>71</v>
       </c>
       <c r="E13" t="s">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="F13" t="s">
-        <v>102</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B14" t="s">
-        <v>85</v>
+        <v>21</v>
       </c>
       <c r="C14" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D14" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E14" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="F14" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C15" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D15" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B16" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="C16" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D16" t="s">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E16" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="F16" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="C17" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D17" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E17" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="F17" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="C18" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D18" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E18" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="F18" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="C19" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D19" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E19" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="F19" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D20" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E20" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="F20" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="C21" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D21" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="E21" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="F21" t="s">
-        <v>104</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>32</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="3">
-        <v>45836</v>
+        <v>45838</v>
       </c>
       <c r="D22" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="E22" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="F22" t="s">
-        <v>105</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="C23" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D23" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="E23" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="F23" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D24" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="E24" t="s">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="F24" t="s">
-        <v>91</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C25" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D25" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E25" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F25" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C26" s="3">
-        <v>45835</v>
+        <v>45838</v>
       </c>
       <c r="D26" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="E26" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="F26" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" t="s">
-        <v>68</v>
-      </c>
-      <c r="B27" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D27" t="s">
-        <v>91</v>
-      </c>
-      <c r="E27" t="s">
-        <v>98</v>
-      </c>
-      <c r="F27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6">
-      <c r="A28" t="s">
-        <v>69</v>
-      </c>
-      <c r="B28" t="s">
-        <v>20</v>
-      </c>
-      <c r="C28" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D28" t="s">
-        <v>91</v>
-      </c>
-      <c r="E28" t="s">
-        <v>98</v>
-      </c>
-      <c r="F28" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6">
-      <c r="A29" t="s">
-        <v>70</v>
-      </c>
-      <c r="B29" t="s">
-        <v>86</v>
-      </c>
-      <c r="C29" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D29" t="s">
-        <v>91</v>
-      </c>
-      <c r="E29" t="s">
-        <v>98</v>
-      </c>
-      <c r="F29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6">
-      <c r="A30" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30" t="s">
-        <v>20</v>
-      </c>
-      <c r="C30" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D30" t="s">
-        <v>91</v>
-      </c>
-      <c r="E30" t="s">
-        <v>98</v>
-      </c>
-      <c r="F30" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6">
-      <c r="A31" t="s">
-        <v>35</v>
-      </c>
-      <c r="B31" t="s">
-        <v>20</v>
-      </c>
-      <c r="C31" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D31" t="s">
-        <v>91</v>
-      </c>
-      <c r="E31" t="s">
-        <v>98</v>
-      </c>
-      <c r="F31" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6">
-      <c r="A32" t="s">
-        <v>71</v>
-      </c>
-      <c r="B32" t="s">
-        <v>20</v>
-      </c>
-      <c r="C32" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D32" t="s">
-        <v>91</v>
-      </c>
-      <c r="E32" t="s">
-        <v>99</v>
-      </c>
-      <c r="F32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6">
-      <c r="A33" t="s">
-        <v>72</v>
-      </c>
-      <c r="B33" t="s">
-        <v>20</v>
-      </c>
-      <c r="C33" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D33" t="s">
-        <v>91</v>
-      </c>
-      <c r="E33" t="s">
-        <v>99</v>
-      </c>
-      <c r="F33" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6">
-      <c r="A34" t="s">
-        <v>73</v>
-      </c>
-      <c r="B34" t="s">
-        <v>20</v>
-      </c>
-      <c r="C34" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D34" t="s">
-        <v>91</v>
-      </c>
-      <c r="E34" t="s">
-        <v>99</v>
-      </c>
-      <c r="F34" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6">
-      <c r="A35" t="s">
-        <v>74</v>
-      </c>
-      <c r="B35" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D35" t="s">
-        <v>91</v>
-      </c>
-      <c r="E35" t="s">
-        <v>99</v>
-      </c>
-      <c r="F35" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6">
-      <c r="A36" t="s">
         <v>75</v>
-      </c>
-      <c r="B36" t="s">
-        <v>20</v>
-      </c>
-      <c r="C36" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D36" t="s">
-        <v>91</v>
-      </c>
-      <c r="E36" t="s">
-        <v>99</v>
-      </c>
-      <c r="F36" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" t="s">
-        <v>76</v>
-      </c>
-      <c r="B37" t="s">
-        <v>20</v>
-      </c>
-      <c r="C37" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D37" t="s">
-        <v>91</v>
-      </c>
-      <c r="E37" t="s">
-        <v>99</v>
-      </c>
-      <c r="F37" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" t="s">
-        <v>77</v>
-      </c>
-      <c r="B38" t="s">
-        <v>20</v>
-      </c>
-      <c r="C38" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D38" t="s">
-        <v>91</v>
-      </c>
-      <c r="E38" t="s">
-        <v>99</v>
-      </c>
-      <c r="F38" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39" t="s">
-        <v>20</v>
-      </c>
-      <c r="C39" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D39" t="s">
-        <v>91</v>
-      </c>
-      <c r="E39" t="s">
-        <v>99</v>
-      </c>
-      <c r="F39" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" t="s">
-        <v>79</v>
-      </c>
-      <c r="B40" t="s">
-        <v>20</v>
-      </c>
-      <c r="C40" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D40" t="s">
-        <v>91</v>
-      </c>
-      <c r="E40" t="s">
-        <v>99</v>
-      </c>
-      <c r="F40" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" t="s">
-        <v>20</v>
-      </c>
-      <c r="C41" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D41" t="s">
-        <v>91</v>
-      </c>
-      <c r="E41" t="s">
-        <v>99</v>
-      </c>
-      <c r="F41" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" t="s">
-        <v>81</v>
-      </c>
-      <c r="B42" t="s">
-        <v>20</v>
-      </c>
-      <c r="C42" s="3">
-        <v>45836</v>
-      </c>
-      <c r="D42" t="s">
-        <v>91</v>
-      </c>
-      <c r="E42" t="s">
-        <v>99</v>
-      </c>
-      <c r="F42" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" t="s">
-        <v>82</v>
-      </c>
-      <c r="B43" t="s">
-        <v>20</v>
-      </c>
-      <c r="C43" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D43" t="s">
-        <v>91</v>
-      </c>
-      <c r="E43" t="s">
-        <v>98</v>
-      </c>
-      <c r="F43" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6">
-      <c r="A44" t="s">
-        <v>83</v>
-      </c>
-      <c r="B44" t="s">
-        <v>20</v>
-      </c>
-      <c r="C44" s="3">
-        <v>45835</v>
-      </c>
-      <c r="D44" t="s">
-        <v>91</v>
-      </c>
-      <c r="E44" t="s">
-        <v>98</v>
-      </c>
-      <c r="F44" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45" t="s">
-        <v>29</v>
-      </c>
-      <c r="B45" t="s">
-        <v>20</v>
-      </c>
-      <c r="C45" s="3">
-        <v>45836</v>
-      </c>
-      <c r="D45" t="s">
-        <v>91</v>
-      </c>
-      <c r="E45" t="s">
-        <v>98</v>
-      </c>
-      <c r="F45" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated load files for 7.2.25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="110">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (06/30/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (06/30/2025)</t>
+    <t>Adoptions (07/01/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (07/01/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -104,13 +104,13 @@
     <t>Review Date</t>
   </si>
   <si>
-    <t>A0058803379</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Cat Isolation 231, Cage 6</t>
-  </si>
-  <si>
-    <t>2025-07-02</t>
+    <t>A0058819245</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Adoption Condo Rooms, Rabbitat 2</t>
+  </si>
+  <si>
+    <t>2025-07-08</t>
   </si>
   <si>
     <t>A0058812302</t>
@@ -149,87 +149,90 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058563467</t>
-  </si>
-  <si>
-    <t>A0058772179</t>
-  </si>
-  <si>
-    <t>A0058816447</t>
-  </si>
-  <si>
-    <t>A0015599570</t>
-  </si>
-  <si>
-    <t>A0054021734</t>
-  </si>
-  <si>
-    <t>A0058804211</t>
-  </si>
-  <si>
-    <t>A0058811219</t>
-  </si>
-  <si>
-    <t>A0058812472</t>
-  </si>
-  <si>
-    <t>A0058812728</t>
-  </si>
-  <si>
-    <t>A0058813263</t>
-  </si>
-  <si>
-    <t>A0058813495</t>
-  </si>
-  <si>
-    <t>A0058817552</t>
-  </si>
-  <si>
-    <t>A0058501223</t>
-  </si>
-  <si>
-    <t>A0058814043</t>
-  </si>
-  <si>
-    <t>A0058814049</t>
-  </si>
-  <si>
-    <t>A0058814052</t>
-  </si>
-  <si>
-    <t>A0058814056</t>
-  </si>
-  <si>
-    <t>A0058814060</t>
-  </si>
-  <si>
-    <t>A0058817102</t>
-  </si>
-  <si>
-    <t>A0058811036</t>
-  </si>
-  <si>
-    <t>A0058816089</t>
-  </si>
-  <si>
-    <t>A0058811183</t>
-  </si>
-  <si>
-    <t>A0058811207</t>
+    <t>A0058735803</t>
+  </si>
+  <si>
+    <t>A0058775077</t>
+  </si>
+  <si>
+    <t>A0058811083</t>
+  </si>
+  <si>
+    <t>A0058820045</t>
+  </si>
+  <si>
+    <t>A0058822904</t>
+  </si>
+  <si>
+    <t>A0058822907</t>
+  </si>
+  <si>
+    <t>A0058822909</t>
+  </si>
+  <si>
+    <t>A0058822916</t>
+  </si>
+  <si>
+    <t>A0058301744</t>
+  </si>
+  <si>
+    <t>A0058819858</t>
+  </si>
+  <si>
+    <t>A0058819243</t>
+  </si>
+  <si>
+    <t>A0058819386</t>
+  </si>
+  <si>
+    <t>A0058820115</t>
+  </si>
+  <si>
+    <t>A0058821278</t>
+  </si>
+  <si>
+    <t>A0058821500</t>
+  </si>
+  <si>
+    <t>A0058821514</t>
+  </si>
+  <si>
+    <t>A0058821534</t>
+  </si>
+  <si>
+    <t>A0058821547</t>
+  </si>
+  <si>
+    <t>A0058822625</t>
+  </si>
+  <si>
+    <t>A0058823210</t>
+  </si>
+  <si>
+    <t>A0058823213</t>
+  </si>
+  <si>
+    <t>A0058823216</t>
+  </si>
+  <si>
+    <t>A0058823219</t>
+  </si>
+  <si>
+    <t>A0058815706</t>
+  </si>
+  <si>
+    <t>A0058815714</t>
+  </si>
+  <si>
+    <t>A0058815755</t>
+  </si>
+  <si>
+    <t>A0058815762</t>
   </si>
   <si>
     <t>Rabbit</t>
   </si>
   <si>
-    <t>Domestic (Cage) Bird</t>
-  </si>
-  <si>
-    <t>Farm Type Fowl</t>
-  </si>
-  <si>
-    <t>Clinic</t>
-  </si>
-  <si>
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
@@ -245,97 +248,91 @@
     <t>Transfer In</t>
   </si>
   <si>
-    <t>Retention</t>
+    <t>Evaluation/Poss Adopt - OTC!</t>
   </si>
   <si>
     <t>Euthanasia Request - OTC!</t>
   </si>
   <si>
+    <t>Evaluation/Poss Adopt - FIELD!</t>
+  </si>
+  <si>
+    <t>Medical Treatment - OTC!</t>
+  </si>
+  <si>
+    <t>Signed Over</t>
+  </si>
+  <si>
+    <t>OTC</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>Feral Cat Focus</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
     <t>DOA</t>
   </si>
   <si>
-    <t>Guardian Surrender - OTC!</t>
-  </si>
-  <si>
-    <t>OTC</t>
-  </si>
-  <si>
-    <t>Guardian Surrender - FIELD!</t>
-  </si>
-  <si>
-    <t>Owned More than 30 Days FIELD!</t>
-  </si>
-  <si>
-    <t>Signed Over</t>
-  </si>
-  <si>
-    <t>Owner died</t>
-  </si>
-  <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>ACO or DCO in County</t>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Seized – Cruelty</t>
+  </si>
+  <si>
+    <t>Seized – General</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
+    <t>Seized – Eviction</t>
+  </si>
+  <si>
+    <t>Seized – Police</t>
+  </si>
+  <si>
+    <t>Seized – Owner Died</t>
+  </si>
+  <si>
+    <t>Seized – Order Violation</t>
+  </si>
+  <si>
+    <t>Seized - Hoarding</t>
+  </si>
+  <si>
+    <t>OTC - OS - SAFE</t>
+  </si>
+  <si>
+    <t>Clinic - Medical Treatment</t>
+  </si>
+  <si>
+    <t>Clinic - Stray</t>
   </si>
   <si>
     <t>Clinic - Retention</t>
-  </si>
-  <si>
-    <t>Clinic - Stray</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Seized – Owner Died</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
-  </si>
-  <si>
-    <t>Seized – Cruelty</t>
-  </si>
-  <si>
-    <t>Seized – General</t>
-  </si>
-  <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
-    <t>Seized – Eviction</t>
-  </si>
-  <si>
-    <t>Seized – Police</t>
-  </si>
-  <si>
-    <t>Seized – Order Violation</t>
-  </si>
-  <si>
-    <t>Seized - Hoarding</t>
-  </si>
-  <si>
-    <t>OTC - OS - SAFE</t>
-  </si>
-  <si>
-    <t>Clinic - Medical Treatment</t>
   </si>
   <si>
     <t>Clinic - Case Assistance</t>
@@ -744,7 +741,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -752,7 +749,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -768,7 +765,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -808,7 +805,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>8</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -824,7 +821,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>18</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -832,7 +829,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -856,7 +853,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -875,10 +872,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C20">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -886,10 +883,10 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C21">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -897,10 +894,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="C22">
-        <v>146</v>
+        <v>129</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -908,7 +905,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C23">
         <v>26</v>
@@ -919,7 +916,7 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C24">
         <v>0</v>
@@ -930,10 +927,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>163</v>
+        <v>187</v>
       </c>
       <c r="C25">
-        <v>218</v>
+        <v>202</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -982,7 +979,7 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>20</v>
@@ -996,125 +993,110 @@
     </row>
     <row r="34" spans="1:4">
       <c r="A34" t="s">
-        <v>75</v>
-      </c>
-      <c r="C34">
-        <v>2</v>
+        <v>76</v>
+      </c>
+      <c r="B34">
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" t="s">
-        <v>78</v>
-      </c>
-      <c r="B35">
-        <v>2</v>
-      </c>
-      <c r="C35">
-        <v>2</v>
-      </c>
-      <c r="D35">
-        <v>1</v>
+        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>89</v>
-      </c>
-      <c r="B36">
+        <v>86</v>
+      </c>
+      <c r="C36">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>94</v>
-      </c>
-      <c r="B38">
-        <v>1</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="C39">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>92</v>
-      </c>
-      <c r="D44">
-        <v>5</v>
+        <v>88</v>
+      </c>
+      <c r="B44">
+        <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>93</v>
-      </c>
-      <c r="B47">
-        <v>1</v>
+        <v>99</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>72</v>
-      </c>
-      <c r="C50">
+        <v>73</v>
+      </c>
+      <c r="B50">
         <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B51">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D51">
         <v>2</v>
@@ -1122,59 +1104,53 @@
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>90</v>
-      </c>
-      <c r="B52">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="C52">
+        <v>2</v>
+      </c>
+      <c r="D52">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>88</v>
-      </c>
-      <c r="B55">
-        <v>1</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>87</v>
-      </c>
-      <c r="D56">
-        <v>2</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1184,7 +1160,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1212,19 +1188,19 @@
         <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C2" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1232,19 +1208,19 @@
         <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="C3" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1252,19 +1228,19 @@
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1272,19 +1248,19 @@
         <v>47</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F5" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1292,19 +1268,19 @@
         <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F6" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1312,19 +1288,19 @@
         <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1332,19 +1308,19 @@
         <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C8" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D8" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E8" t="s">
         <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -1352,19 +1328,19 @@
         <v>51</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C9" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F9" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -1372,19 +1348,19 @@
         <v>52</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="E10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -1392,19 +1368,19 @@
         <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D11" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="E11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="F11" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -1412,276 +1388,276 @@
         <v>54</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="C12" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D12" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F12" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>71</v>
       </c>
       <c r="C13" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D13" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F13" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D14" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F14" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="C15" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D15" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E15" t="s">
         <v>83</v>
       </c>
       <c r="F15" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D16" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E16" t="s">
         <v>83</v>
       </c>
       <c r="F16" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="C17" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D17" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E17" t="s">
         <v>83</v>
       </c>
       <c r="F17" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="C18" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E18" t="s">
         <v>83</v>
       </c>
       <c r="F18" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="C19" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D19" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E19" t="s">
         <v>83</v>
       </c>
       <c r="F19" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D20" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F20" t="s">
-        <v>93</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="C21" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E21" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F21" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F22" t="s">
-        <v>94</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="C23" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E23" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B24" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D24" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E24" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="F24" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C25" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D25" t="s">
         <v>75</v>
       </c>
       <c r="E25" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="F25" t="s">
         <v>75</v>
@@ -1689,22 +1665,82 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C26" s="3">
-        <v>45838</v>
+        <v>45839</v>
       </c>
       <c r="D26" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E26" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F26" t="s">
-        <v>75</v>
+        <v>76</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="3">
+        <v>45839</v>
+      </c>
+      <c r="D27" t="s">
+        <v>76</v>
+      </c>
+      <c r="E27" t="s">
+        <v>84</v>
+      </c>
+      <c r="F27" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>69</v>
+      </c>
+      <c r="B28" t="s">
+        <v>20</v>
+      </c>
+      <c r="C28" s="3">
+        <v>45839</v>
+      </c>
+      <c r="D28" t="s">
+        <v>76</v>
+      </c>
+      <c r="E28" t="s">
+        <v>84</v>
+      </c>
+      <c r="F28" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" t="s">
+        <v>20</v>
+      </c>
+      <c r="C29" s="3">
+        <v>45839</v>
+      </c>
+      <c r="D29" t="s">
+        <v>76</v>
+      </c>
+      <c r="E29" t="s">
+        <v>84</v>
+      </c>
+      <c r="F29" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 7/7/25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="133">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (07/01/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (07/01/2025)</t>
+    <t>Adoptions (07/03/2025, 07/05/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (07/03/2025, 07/05/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -104,31 +104,43 @@
     <t>Review Date</t>
   </si>
   <si>
+    <t>A0058840701</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Isolation 231, Cage 4</t>
+  </si>
+  <si>
+    <t>2025-07-08</t>
+  </si>
+  <si>
+    <t>A0058839495</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Isolation 234, Cage 6</t>
+  </si>
+  <si>
+    <t>A0058812861</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 2</t>
+  </si>
+  <si>
+    <t>2025-07-07</t>
+  </si>
+  <si>
+    <t>A0058849616</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Multi Animal Holding</t>
+  </si>
+  <si>
+    <t>2025-07-11</t>
+  </si>
+  <si>
     <t>A0058819245</t>
   </si>
   <si>
-    <t xml:space="preserve">  Cat Adoption Condo Rooms, Rabbitat 2</t>
-  </si>
-  <si>
-    <t>2025-07-08</t>
-  </si>
-  <si>
-    <t>A0058812302</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  ICU, 01</t>
-  </si>
-  <si>
-    <t>2025-07-05</t>
-  </si>
-  <si>
-    <t>A0058812861</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Rabbitat 2</t>
-  </si>
-  <si>
-    <t>2025-07-07</t>
+    <t xml:space="preserve">  Small Animals &amp; Exotics, Mammal 4</t>
   </si>
   <si>
     <t>AnimalNumber</t>
@@ -149,88 +161,136 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058735803</t>
-  </si>
-  <si>
-    <t>A0058775077</t>
-  </si>
-  <si>
-    <t>A0058811083</t>
-  </si>
-  <si>
-    <t>A0058820045</t>
-  </si>
-  <si>
-    <t>A0058822904</t>
-  </si>
-  <si>
-    <t>A0058822907</t>
-  </si>
-  <si>
-    <t>A0058822909</t>
-  </si>
-  <si>
-    <t>A0058822916</t>
-  </si>
-  <si>
-    <t>A0058301744</t>
-  </si>
-  <si>
-    <t>A0058819858</t>
-  </si>
-  <si>
-    <t>A0058819243</t>
-  </si>
-  <si>
-    <t>A0058819386</t>
-  </si>
-  <si>
-    <t>A0058820115</t>
-  </si>
-  <si>
-    <t>A0058821278</t>
-  </si>
-  <si>
-    <t>A0058821500</t>
-  </si>
-  <si>
-    <t>A0058821514</t>
-  </si>
-  <si>
-    <t>A0058821534</t>
-  </si>
-  <si>
-    <t>A0058821547</t>
-  </si>
-  <si>
-    <t>A0058822625</t>
-  </si>
-  <si>
-    <t>A0058823210</t>
-  </si>
-  <si>
-    <t>A0058823213</t>
-  </si>
-  <si>
-    <t>A0058823216</t>
-  </si>
-  <si>
-    <t>A0058823219</t>
-  </si>
-  <si>
-    <t>A0058815706</t>
-  </si>
-  <si>
-    <t>A0058815714</t>
-  </si>
-  <si>
-    <t>A0058815755</t>
-  </si>
-  <si>
-    <t>A0058815762</t>
-  </si>
-  <si>
-    <t>Rabbit</t>
+    <t>A0058837698</t>
+  </si>
+  <si>
+    <t>A0054633714</t>
+  </si>
+  <si>
+    <t>A0058797381</t>
+  </si>
+  <si>
+    <t>A0058797603</t>
+  </si>
+  <si>
+    <t>A0058797608</t>
+  </si>
+  <si>
+    <t>A0058797612</t>
+  </si>
+  <si>
+    <t>A0058797613</t>
+  </si>
+  <si>
+    <t>A0058797614</t>
+  </si>
+  <si>
+    <t>A0058797617</t>
+  </si>
+  <si>
+    <t>A0058828034</t>
+  </si>
+  <si>
+    <t>A0058828077</t>
+  </si>
+  <si>
+    <t>A0058829525</t>
+  </si>
+  <si>
+    <t>A0058840714</t>
+  </si>
+  <si>
+    <t>A0058840716</t>
+  </si>
+  <si>
+    <t>A0058846483</t>
+  </si>
+  <si>
+    <t>A0058849219</t>
+  </si>
+  <si>
+    <t>A0055874744</t>
+  </si>
+  <si>
+    <t>A0058421981</t>
+  </si>
+  <si>
+    <t>A0058836708</t>
+  </si>
+  <si>
+    <t>A0058840216</t>
+  </si>
+  <si>
+    <t>A0058840227</t>
+  </si>
+  <si>
+    <t>A0058840242</t>
+  </si>
+  <si>
+    <t>A0058840248</t>
+  </si>
+  <si>
+    <t>A0058840262</t>
+  </si>
+  <si>
+    <t>A0058849570</t>
+  </si>
+  <si>
+    <t>A0058823724</t>
+  </si>
+  <si>
+    <t>A0058823725</t>
+  </si>
+  <si>
+    <t>A0058823726</t>
+  </si>
+  <si>
+    <t>A0058828052</t>
+  </si>
+  <si>
+    <t>A0058828053</t>
+  </si>
+  <si>
+    <t>A0058836765</t>
+  </si>
+  <si>
+    <t>A0058837850</t>
+  </si>
+  <si>
+    <t>A0058838635</t>
+  </si>
+  <si>
+    <t>A0058838653</t>
+  </si>
+  <si>
+    <t>A0058838661</t>
+  </si>
+  <si>
+    <t>A0058838669</t>
+  </si>
+  <si>
+    <t>A0058847120</t>
+  </si>
+  <si>
+    <t>A0058847793</t>
+  </si>
+  <si>
+    <t>A0058848390</t>
+  </si>
+  <si>
+    <t>A0058848924</t>
+  </si>
+  <si>
+    <t>A0058067302</t>
+  </si>
+  <si>
+    <t>A0058838875</t>
+  </si>
+  <si>
+    <t>Domestic (Cage) Bird</t>
+  </si>
+  <si>
+    <t>Clinic</t>
   </si>
   <si>
     <t>Owner/Guardian Surrender</t>
@@ -248,54 +308,66 @@
     <t>Transfer In</t>
   </si>
   <si>
+    <t>Euthanasia Request - OTC!</t>
+  </si>
+  <si>
+    <t>Euthanasia Request - FIELD!</t>
+  </si>
+  <si>
     <t>Evaluation/Poss Adopt - OTC!</t>
   </si>
   <si>
-    <t>Euthanasia Request - OTC!</t>
-  </si>
-  <si>
-    <t>Evaluation/Poss Adopt - FIELD!</t>
-  </si>
-  <si>
-    <t>Medical Treatment - OTC!</t>
+    <t>Guardian Surrender - OTC!</t>
+  </si>
+  <si>
+    <t>DOA</t>
+  </si>
+  <si>
+    <t>Owned More than 30 Days - OTC!</t>
+  </si>
+  <si>
+    <t>Owned 30 Days or Less - OTC!</t>
   </si>
   <si>
     <t>Signed Over</t>
   </si>
   <si>
+    <t>No Hold</t>
+  </si>
+  <si>
     <t>OTC</t>
   </si>
   <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>Feral Cat Focus</t>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>ACO or DCO in County</t>
+  </si>
+  <si>
+    <t>Clinic - Stray</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
   </si>
   <si>
     <t>OTC – OS</t>
   </si>
   <si>
-    <t>Euthanasia Request</t>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
   </si>
   <si>
     <t>Field – OS</t>
   </si>
   <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
     <t>Seized – Abandoned</t>
   </si>
   <si>
@@ -327,9 +399,6 @@
   </si>
   <si>
     <t>Clinic - Medical Treatment</t>
-  </si>
-  <si>
-    <t>Clinic - Stray</t>
   </si>
   <si>
     <t>Clinic - Retention</t>
@@ -721,7 +790,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -741,7 +810,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>17</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -749,7 +818,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -765,7 +834,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>188</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -781,7 +850,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -805,7 +874,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>26</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -821,7 +890,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -829,7 +898,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>11</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -853,7 +922,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -872,10 +941,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C20">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -883,10 +952,10 @@
         <v>21</v>
       </c>
       <c r="B21">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C21">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -894,10 +963,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="C22">
-        <v>129</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -905,10 +974,10 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C23">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -916,10 +985,10 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C24">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -927,10 +996,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>187</v>
+        <v>156</v>
       </c>
       <c r="C25">
-        <v>202</v>
+        <v>245</v>
       </c>
     </row>
     <row r="27" spans="1:3">
@@ -963,194 +1032,234 @@
         <v>33</v>
       </c>
       <c r="C29" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
         <v>35</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>36</v>
       </c>
-      <c r="C30" t="s">
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="33" spans="1:4">
-      <c r="A33" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C33" s="1" t="s">
+      <c r="B31" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
+      <c r="A35" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D35" s="1" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" t="s">
-        <v>76</v>
-      </c>
-      <c r="B34">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="C36">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" t="s">
-        <v>91</v>
+        <v>101</v>
+      </c>
+      <c r="B37">
+        <v>2</v>
+      </c>
+      <c r="C37">
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>92</v>
+        <v>110</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="C39">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" t="s">
-        <v>93</v>
+        <v>114</v>
+      </c>
+      <c r="B40">
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" t="s">
-        <v>94</v>
+        <v>116</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" t="s">
-        <v>95</v>
+        <v>117</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" t="s">
-        <v>96</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" t="s">
-        <v>88</v>
-      </c>
-      <c r="B44">
-        <v>1</v>
+        <v>119</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" t="s">
-        <v>98</v>
+        <v>113</v>
+      </c>
+      <c r="B46">
+        <v>6</v>
+      </c>
+      <c r="C46">
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" t="s">
-        <v>99</v>
+        <v>121</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>101</v>
+        <v>123</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>73</v>
-      </c>
-      <c r="B50">
-        <v>1</v>
+        <v>124</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>75</v>
-      </c>
-      <c r="B51">
-        <v>12</v>
-      </c>
-      <c r="D51">
-        <v>2</v>
+        <v>125</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>85</v>
+        <v>93</v>
+      </c>
+      <c r="B52">
+        <v>1</v>
       </c>
       <c r="C52">
-        <v>2</v>
-      </c>
-      <c r="D52">
         <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>95</v>
+      </c>
+      <c r="B53">
+        <v>16</v>
+      </c>
+      <c r="D53">
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>103</v>
+        <v>112</v>
+      </c>
+      <c r="B54">
+        <v>9</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>104</v>
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>105</v>
+        <v>127</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>106</v>
+        <v>109</v>
+      </c>
+      <c r="B57">
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>128</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>108</v>
+        <v>129</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" t="s">
-        <v>109</v>
+        <v>130</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1160,587 +1269,927 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D2" t="s">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="E2" t="s">
-        <v>77</v>
+        <v>95</v>
       </c>
       <c r="F2" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="F3" t="s">
-        <v>85</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E4" t="s">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="F4" t="s">
-        <v>85</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D5" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="F5" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E6" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E7" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="F7" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D8" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E8" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="F8" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D9" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E9" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
       <c r="F9" t="s">
-        <v>87</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
         <v>20</v>
       </c>
       <c r="C10" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D10" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="E10" t="s">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="F10" t="s">
-        <v>73</v>
+        <v>112</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>20</v>
       </c>
       <c r="C11" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D11" t="s">
-        <v>74</v>
+        <v>92</v>
       </c>
       <c r="E11" t="s">
-        <v>81</v>
+        <v>100</v>
       </c>
       <c r="F11" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>21</v>
       </c>
       <c r="C12" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D12" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E12" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="F12" t="s">
-        <v>75</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>59</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
       <c r="C13" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D13" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E13" t="s">
-        <v>82</v>
+        <v>101</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B14" t="s">
         <v>20</v>
       </c>
       <c r="C14" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D14" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="F14" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B15" t="s">
         <v>20</v>
       </c>
       <c r="C15" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D15" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
       <c r="F15" t="s">
-        <v>75</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B16" t="s">
         <v>20</v>
       </c>
       <c r="C16" s="3">
-        <v>45839</v>
+        <v>45843</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E16" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="F16" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="3">
-        <v>45839</v>
+        <v>45843</v>
       </c>
       <c r="D17" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="E17" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="F17" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B18" t="s">
         <v>20</v>
       </c>
       <c r="C18" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>102</v>
       </c>
       <c r="F18" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C19" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D19" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>83</v>
+        <v>103</v>
       </c>
       <c r="F19" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D20" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E20" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D21" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E21" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F21" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D22" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E22" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F22" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B23" t="s">
         <v>20</v>
       </c>
       <c r="C23" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D23" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E23" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F23" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B24" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D24" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E24" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F24" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B25" t="s">
         <v>20</v>
       </c>
       <c r="C25" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D25" t="s">
-        <v>75</v>
+        <v>94</v>
       </c>
       <c r="E25" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="F25" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C26" s="3">
-        <v>45839</v>
+        <v>45843</v>
       </c>
       <c r="D26" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="E26" t="s">
-        <v>84</v>
+        <v>104</v>
       </c>
       <c r="F26" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B27" t="s">
         <v>20</v>
       </c>
       <c r="C27" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D27" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="E27" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="F27" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B28" t="s">
         <v>20</v>
       </c>
       <c r="C28" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D28" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="E28" t="s">
-        <v>84</v>
+        <v>105</v>
       </c>
       <c r="F28" t="s">
-        <v>76</v>
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
         <v>20</v>
       </c>
       <c r="C29" s="3">
-        <v>45839</v>
+        <v>45841</v>
       </c>
       <c r="D29" t="s">
+        <v>95</v>
+      </c>
+      <c r="E29" t="s">
+        <v>105</v>
+      </c>
+      <c r="F29" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" t="s">
         <v>76</v>
       </c>
-      <c r="E29" t="s">
+      <c r="B30" t="s">
+        <v>20</v>
+      </c>
+      <c r="C30" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D30" t="s">
+        <v>95</v>
+      </c>
+      <c r="E30" t="s">
+        <v>105</v>
+      </c>
+      <c r="F30" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D31" t="s">
+        <v>95</v>
+      </c>
+      <c r="E31" t="s">
+        <v>105</v>
+      </c>
+      <c r="F31" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" t="s">
+        <v>20</v>
+      </c>
+      <c r="C32" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D32" t="s">
+        <v>95</v>
+      </c>
+      <c r="E32" t="s">
+        <v>105</v>
+      </c>
+      <c r="F32" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D33" t="s">
+        <v>95</v>
+      </c>
+      <c r="E33" t="s">
+        <v>105</v>
+      </c>
+      <c r="F33" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" t="s">
+        <v>80</v>
+      </c>
+      <c r="B34" t="s">
+        <v>20</v>
+      </c>
+      <c r="C34" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D34" t="s">
+        <v>95</v>
+      </c>
+      <c r="E34" t="s">
+        <v>106</v>
+      </c>
+      <c r="F34" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" t="s">
+        <v>81</v>
+      </c>
+      <c r="B35" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D35" t="s">
+        <v>95</v>
+      </c>
+      <c r="E35" t="s">
+        <v>106</v>
+      </c>
+      <c r="F35" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6">
+      <c r="A36" t="s">
+        <v>82</v>
+      </c>
+      <c r="B36" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D36" t="s">
+        <v>95</v>
+      </c>
+      <c r="E36" t="s">
+        <v>106</v>
+      </c>
+      <c r="F36" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" t="s">
+        <v>83</v>
+      </c>
+      <c r="B37" t="s">
+        <v>20</v>
+      </c>
+      <c r="C37" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D37" t="s">
+        <v>95</v>
+      </c>
+      <c r="E37" t="s">
+        <v>106</v>
+      </c>
+      <c r="F37" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" t="s">
+        <v>20</v>
+      </c>
+      <c r="C38" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D38" t="s">
+        <v>95</v>
+      </c>
+      <c r="E38" t="s">
+        <v>106</v>
+      </c>
+      <c r="F38" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" t="s">
+        <v>29</v>
+      </c>
+      <c r="B39" t="s">
+        <v>20</v>
+      </c>
+      <c r="C39" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D39" t="s">
+        <v>95</v>
+      </c>
+      <c r="E39" t="s">
+        <v>106</v>
+      </c>
+      <c r="F39" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" t="s">
         <v>84</v>
       </c>
-      <c r="F29" t="s">
-        <v>76</v>
+      <c r="B40" t="s">
+        <v>20</v>
+      </c>
+      <c r="C40" s="3">
+        <v>45843</v>
+      </c>
+      <c r="D40" t="s">
+        <v>95</v>
+      </c>
+      <c r="E40" t="s">
+        <v>105</v>
+      </c>
+      <c r="F40" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6">
+      <c r="A41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B41" t="s">
+        <v>20</v>
+      </c>
+      <c r="C41" s="3">
+        <v>45843</v>
+      </c>
+      <c r="D41" t="s">
+        <v>95</v>
+      </c>
+      <c r="E41" t="s">
+        <v>105</v>
+      </c>
+      <c r="F41" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" t="s">
+        <v>86</v>
+      </c>
+      <c r="B42" t="s">
+        <v>20</v>
+      </c>
+      <c r="C42" s="3">
+        <v>45843</v>
+      </c>
+      <c r="D42" t="s">
+        <v>95</v>
+      </c>
+      <c r="E42" t="s">
+        <v>105</v>
+      </c>
+      <c r="F42" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" t="s">
+        <v>87</v>
+      </c>
+      <c r="B43" t="s">
+        <v>20</v>
+      </c>
+      <c r="C43" s="3">
+        <v>45843</v>
+      </c>
+      <c r="D43" t="s">
+        <v>95</v>
+      </c>
+      <c r="E43" t="s">
+        <v>107</v>
+      </c>
+      <c r="F43" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6">
+      <c r="A44" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" t="s">
+        <v>90</v>
+      </c>
+      <c r="C44" s="3">
+        <v>45843</v>
+      </c>
+      <c r="D44" t="s">
+        <v>95</v>
+      </c>
+      <c r="E44" t="s">
+        <v>106</v>
+      </c>
+      <c r="F44" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" t="s">
+        <v>88</v>
+      </c>
+      <c r="B45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D45" t="s">
+        <v>96</v>
+      </c>
+      <c r="E45" t="s">
+        <v>108</v>
+      </c>
+      <c r="F45" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46" t="s">
+        <v>21</v>
+      </c>
+      <c r="C46" s="3">
+        <v>45841</v>
+      </c>
+      <c r="D46" t="s">
+        <v>96</v>
+      </c>
+      <c r="E46" t="s">
+        <v>108</v>
+      </c>
+      <c r="F46" t="s">
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 7/10/25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="102">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (07/08/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (07/08/2025)</t>
+    <t>Adoptions (07/09/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (07/09/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -140,91 +140,133 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0058742107</t>
-  </si>
-  <si>
-    <t>A0058811636</t>
-  </si>
-  <si>
-    <t>A0058819189</t>
-  </si>
-  <si>
-    <t>A0058836833</t>
-  </si>
-  <si>
-    <t>A0058862207</t>
-  </si>
-  <si>
-    <t>A0058864061</t>
-  </si>
-  <si>
-    <t>A0058864064</t>
-  </si>
-  <si>
-    <t>A0058864066</t>
-  </si>
-  <si>
-    <t>A0058864067</t>
-  </si>
-  <si>
-    <t>A0058864070</t>
-  </si>
-  <si>
-    <t>A0058864072</t>
-  </si>
-  <si>
-    <t>A0058866048</t>
-  </si>
-  <si>
-    <t>Rodent</t>
+    <t>A0056924261</t>
+  </si>
+  <si>
+    <t>A0058832269</t>
+  </si>
+  <si>
+    <t>A0058862375</t>
+  </si>
+  <si>
+    <t>A0058872179</t>
+  </si>
+  <si>
+    <t>A0058872186</t>
+  </si>
+  <si>
+    <t>A0058873095</t>
+  </si>
+  <si>
+    <t>A0058865640</t>
+  </si>
+  <si>
+    <t>A0058871542</t>
+  </si>
+  <si>
+    <t>A0058872784</t>
+  </si>
+  <si>
+    <t>A0058872788</t>
+  </si>
+  <si>
+    <t>A0058872790</t>
+  </si>
+  <si>
+    <t>A0058872792</t>
+  </si>
+  <si>
+    <t>A0058872796</t>
+  </si>
+  <si>
+    <t>A0058872798</t>
+  </si>
+  <si>
+    <t>A0058872803</t>
+  </si>
+  <si>
+    <t>A0058872805</t>
+  </si>
+  <si>
+    <t>A0058872807</t>
+  </si>
+  <si>
+    <t>A0058872864</t>
+  </si>
+  <si>
+    <t>A0058872867</t>
+  </si>
+  <si>
+    <t>A0058874744</t>
+  </si>
+  <si>
+    <t>A0058874847</t>
+  </si>
+  <si>
+    <t>A0058874851</t>
+  </si>
+  <si>
+    <t>A0058874852</t>
+  </si>
+  <si>
+    <t>A0058874853</t>
+  </si>
+  <si>
+    <t>A0058874855</t>
+  </si>
+  <si>
+    <t>A0058875207</t>
+  </si>
+  <si>
+    <t>Rabbit</t>
   </si>
   <si>
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
+    <t>Seized / Custody</t>
+  </si>
+  <si>
     <t>Stray</t>
   </si>
   <si>
+    <t>Guardian Surrender - OTC!</t>
+  </si>
+  <si>
+    <t>Euthanasia Request - FIELD!</t>
+  </si>
+  <si>
+    <t>DOA</t>
+  </si>
+  <si>
+    <t>Abandoned</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Euthanasia Req – Field</t>
+  </si>
+  <si>
+    <t>Seized – Abandoned</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
+  </si>
+  <si>
     <t>Transfer In</t>
   </si>
   <si>
-    <t>Evaluation/Poss Adopt - OTC!</t>
-  </si>
-  <si>
-    <t>Euthanasia Request - OTC!</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>OTC</t>
-  </si>
-  <si>
-    <t>ACO or DCO in County</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
     <t>Euthanasia Request</t>
   </si>
   <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>DOA</t>
-  </si>
-  <si>
-    <t>Euthanasia Req – Field</t>
-  </si>
-  <si>
     <t>Field – Stray</t>
   </si>
   <si>
     <t>Field – OS</t>
-  </si>
-  <si>
-    <t>Seized – Abandoned</t>
   </si>
   <si>
     <t>Seized – Cruelty</t>
@@ -675,7 +717,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -699,7 +741,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -707,7 +749,7 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -715,7 +757,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -723,7 +765,7 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -739,7 +781,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -755,7 +797,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -763,7 +805,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -771,7 +813,7 @@
         <v>14</v>
       </c>
       <c r="B15">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:2">
@@ -779,7 +821,7 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -787,7 +829,7 @@
         <v>16</v>
       </c>
       <c r="B17">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -806,10 +848,10 @@
         <v>20</v>
       </c>
       <c r="B20">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C20">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -828,10 +870,10 @@
         <v>22</v>
       </c>
       <c r="B22">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C22">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -839,7 +881,7 @@
         <v>23</v>
       </c>
       <c r="B23">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C23">
         <v>27</v>
@@ -850,10 +892,10 @@
         <v>24</v>
       </c>
       <c r="B24">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C24">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -861,10 +903,10 @@
         <v>25</v>
       </c>
       <c r="B25">
-        <v>153</v>
+        <v>164</v>
       </c>
       <c r="C25">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -902,7 +944,7 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="1" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>20</v>
@@ -916,155 +958,158 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33">
-        <v>1</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>65</v>
+        <v>73</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>63</v>
-      </c>
-      <c r="C35">
-        <v>2</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>66</v>
+        <v>77</v>
+      </c>
+      <c r="C36">
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>68</v>
+        <v>83</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>69</v>
+        <v>78</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39">
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>85</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>72</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>73</v>
+        <v>87</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="B50">
-        <v>2</v>
-      </c>
-      <c r="C50">
-        <v>6</v>
+        <v>11</v>
+      </c>
+      <c r="D50">
+        <v>9</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
       <c r="C51">
         <v>1</v>
       </c>
-      <c r="D51">
-        <v>1</v>
-      </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1074,7 +1119,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1102,19 +1147,19 @@
         <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D2" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
       <c r="F2" t="s">
-        <v>62</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1125,16 +1170,16 @@
         <v>21</v>
       </c>
       <c r="C3" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s">
-        <v>57</v>
+        <v>72</v>
       </c>
       <c r="F3" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1142,19 +1187,19 @@
         <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>68</v>
       </c>
       <c r="E4" t="s">
-        <v>58</v>
+        <v>73</v>
       </c>
       <c r="F4" t="s">
-        <v>63</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1162,19 +1207,19 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D5" t="s">
-        <v>54</v>
+        <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="F5" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1185,176 +1230,436 @@
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D6" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>74</v>
       </c>
       <c r="F6" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D7" t="s">
-        <v>55</v>
+        <v>69</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="F7" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D8" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="C10" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F10" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="C11" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D11" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F11" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="C12" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F12" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="C13" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D13" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="E13" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="F13" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>67</v>
       </c>
       <c r="C14" s="3">
-        <v>45846</v>
+        <v>45847</v>
       </c>
       <c r="D14" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" t="s">
+        <v>75</v>
+      </c>
+      <c r="F14" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" t="s">
+        <v>75</v>
+      </c>
+      <c r="F16" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" t="s">
         <v>56</v>
       </c>
-      <c r="E14" t="s">
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" t="s">
+        <v>57</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D18" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" t="s">
+        <v>75</v>
+      </c>
+      <c r="F18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C19" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" t="s">
+        <v>75</v>
+      </c>
+      <c r="F19" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B20" t="s">
+        <v>20</v>
+      </c>
+      <c r="C20" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D20" t="s">
+        <v>70</v>
+      </c>
+      <c r="E20" t="s">
+        <v>75</v>
+      </c>
+      <c r="F20" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D21" t="s">
+        <v>70</v>
+      </c>
+      <c r="E21" t="s">
+        <v>75</v>
+      </c>
+      <c r="F21" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" t="s">
         <v>61</v>
       </c>
-      <c r="F14" t="s">
-        <v>56</v>
+      <c r="B22" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D22" t="s">
+        <v>70</v>
+      </c>
+      <c r="E22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" t="s">
+        <v>20</v>
+      </c>
+      <c r="C23" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D23" t="s">
+        <v>70</v>
+      </c>
+      <c r="E23" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" t="s">
+        <v>63</v>
+      </c>
+      <c r="B24" t="s">
+        <v>20</v>
+      </c>
+      <c r="C24" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D24" t="s">
+        <v>70</v>
+      </c>
+      <c r="E24" t="s">
+        <v>75</v>
+      </c>
+      <c r="F24" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" t="s">
+        <v>64</v>
+      </c>
+      <c r="B25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D25" t="s">
+        <v>70</v>
+      </c>
+      <c r="E25" t="s">
+        <v>75</v>
+      </c>
+      <c r="F25" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C26" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D26" t="s">
+        <v>70</v>
+      </c>
+      <c r="E26" t="s">
+        <v>75</v>
+      </c>
+      <c r="F26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="3">
+        <v>45847</v>
+      </c>
+      <c r="D27" t="s">
+        <v>70</v>
+      </c>
+      <c r="E27" t="s">
+        <v>75</v>
+      </c>
+      <c r="F27" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated files for 7/11/25
</commit_message>
<xml_diff>
--- a/MorningEmail/morning_report.xlsx
+++ b/MorningEmail/morning_report.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="120">
   <si>
     <t>Outcomes</t>
   </si>
@@ -23,10 +23,10 @@
     <t>Count</t>
   </si>
   <si>
-    <t>Adoptions (07/09/2025)</t>
-  </si>
-  <si>
-    <t>If The Fur Fits (07/09/2025)</t>
+    <t>Adoptions (07/10/2025)</t>
+  </si>
+  <si>
+    <t>If The Fur Fits (07/10/2025)</t>
   </si>
   <si>
     <t>Stage</t>
@@ -104,6 +104,15 @@
     <t>Review Date</t>
   </si>
   <si>
+    <t>A0058881800</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Cat Adoption Condo Rooms, Rabbitat 2</t>
+  </si>
+  <si>
+    <t>2025-07-16</t>
+  </si>
+  <si>
     <t>A0058862316</t>
   </si>
   <si>
@@ -122,6 +131,24 @@
     <t>2025-07-11</t>
   </si>
   <si>
+    <t>A0058883107</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Multi-Animal Holding, Room 229, Multi Animal Holding</t>
+  </si>
+  <si>
+    <t>A0058883828</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Receiving, Receiving</t>
+  </si>
+  <si>
+    <t>2025-07-15</t>
+  </si>
+  <si>
+    <t>A0058886564</t>
+  </si>
+  <si>
     <t>AnimalNumber</t>
   </si>
   <si>
@@ -140,147 +167,180 @@
     <t>IntakeGroup</t>
   </si>
   <si>
-    <t>A0056924261</t>
-  </si>
-  <si>
-    <t>A0058832269</t>
-  </si>
-  <si>
-    <t>A0058862375</t>
-  </si>
-  <si>
-    <t>A0058872179</t>
-  </si>
-  <si>
-    <t>A0058872186</t>
-  </si>
-  <si>
-    <t>A0058873095</t>
-  </si>
-  <si>
-    <t>A0058865640</t>
-  </si>
-  <si>
-    <t>A0058871542</t>
-  </si>
-  <si>
-    <t>A0058872784</t>
-  </si>
-  <si>
-    <t>A0058872788</t>
-  </si>
-  <si>
-    <t>A0058872790</t>
-  </si>
-  <si>
-    <t>A0058872792</t>
-  </si>
-  <si>
-    <t>A0058872796</t>
-  </si>
-  <si>
-    <t>A0058872798</t>
-  </si>
-  <si>
-    <t>A0058872803</t>
-  </si>
-  <si>
-    <t>A0058872805</t>
-  </si>
-  <si>
-    <t>A0058872807</t>
-  </si>
-  <si>
-    <t>A0058872864</t>
-  </si>
-  <si>
-    <t>A0058872867</t>
-  </si>
-  <si>
-    <t>A0058874744</t>
-  </si>
-  <si>
-    <t>A0058874847</t>
-  </si>
-  <si>
-    <t>A0058874851</t>
-  </si>
-  <si>
-    <t>A0058874852</t>
-  </si>
-  <si>
-    <t>A0058874853</t>
-  </si>
-  <si>
-    <t>A0058874855</t>
-  </si>
-  <si>
-    <t>A0058875207</t>
+    <t>A0057606326</t>
+  </si>
+  <si>
+    <t>A0057606328</t>
+  </si>
+  <si>
+    <t>A0057606329</t>
+  </si>
+  <si>
+    <t>A0058829471</t>
+  </si>
+  <si>
+    <t>A0058829474</t>
+  </si>
+  <si>
+    <t>A0058847947</t>
+  </si>
+  <si>
+    <t>A0058878916</t>
+  </si>
+  <si>
+    <t>A0058884237</t>
+  </si>
+  <si>
+    <t>A0021403555</t>
+  </si>
+  <si>
+    <t>A0054196266</t>
+  </si>
+  <si>
+    <t>A0058639310</t>
+  </si>
+  <si>
+    <t>A0056617154</t>
+  </si>
+  <si>
+    <t>A0058880548</t>
+  </si>
+  <si>
+    <t>A0058880579</t>
+  </si>
+  <si>
+    <t>A0058880606</t>
+  </si>
+  <si>
+    <t>A0058884959</t>
+  </si>
+  <si>
+    <t>A0058873067</t>
+  </si>
+  <si>
+    <t>A0058873074</t>
+  </si>
+  <si>
+    <t>A0058873076</t>
+  </si>
+  <si>
+    <t>A0058878498</t>
+  </si>
+  <si>
+    <t>A0058880145</t>
+  </si>
+  <si>
+    <t>A0058883197</t>
+  </si>
+  <si>
+    <t>A0058883204</t>
+  </si>
+  <si>
+    <t>A0058883212</t>
+  </si>
+  <si>
+    <t>Domestic (Cage) Bird</t>
   </si>
   <si>
     <t>Rabbit</t>
   </si>
   <si>
+    <t>Reptile/Amphibian</t>
+  </si>
+  <si>
+    <t>Clinic</t>
+  </si>
+  <si>
     <t>Owner/Guardian Surrender</t>
   </si>
   <si>
+    <t>Return</t>
+  </si>
+  <si>
     <t>Seized / Custody</t>
   </si>
   <si>
     <t>Stray</t>
   </si>
   <si>
-    <t>Guardian Surrender - OTC!</t>
-  </si>
-  <si>
-    <t>Euthanasia Request - FIELD!</t>
+    <t>Transfer In</t>
+  </si>
+  <si>
+    <t>Case - Outreach</t>
+  </si>
+  <si>
+    <t>Evaluation/Poss Adopt - OTC!</t>
+  </si>
+  <si>
+    <t>Euthanasia Request - OTC!</t>
+  </si>
+  <si>
+    <t>Owned 30 Days or Less - OTC!</t>
+  </si>
+  <si>
+    <t>Signed Over</t>
+  </si>
+  <si>
+    <t>Hospital</t>
+  </si>
+  <si>
+    <t>Protective Custody</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>No Hold</t>
+  </si>
+  <si>
+    <t>OTC</t>
+  </si>
+  <si>
+    <t>ACO or DCO in County</t>
+  </si>
+  <si>
+    <t>Clinic - Case Assistance - Outreach</t>
+  </si>
+  <si>
+    <t>OTC – OS</t>
+  </si>
+  <si>
+    <t>Euthanasia Request</t>
+  </si>
+  <si>
+    <t>Seized – Signed over</t>
+  </si>
+  <si>
+    <t>Seized – Hospital</t>
+  </si>
+  <si>
+    <t>not counted</t>
+  </si>
+  <si>
+    <t>Field – Stray</t>
+  </si>
+  <si>
+    <t>Intake Count Summary</t>
   </si>
   <si>
     <t>DOA</t>
   </si>
   <si>
-    <t>Abandoned</t>
-  </si>
-  <si>
-    <t>No Hold</t>
-  </si>
-  <si>
-    <t>OTC – OS</t>
-  </si>
-  <si>
     <t>Euthanasia Req – Field</t>
   </si>
   <si>
+    <t>Field – OS</t>
+  </si>
+  <si>
     <t>Seized – Abandoned</t>
   </si>
   <si>
-    <t>Intake Count Summary</t>
-  </si>
-  <si>
-    <t>Transfer In</t>
-  </si>
-  <si>
-    <t>Euthanasia Request</t>
-  </si>
-  <si>
-    <t>Field – Stray</t>
-  </si>
-  <si>
-    <t>Field – OS</t>
-  </si>
-  <si>
     <t>Seized – Cruelty</t>
   </si>
   <si>
     <t>Seized – General</t>
   </si>
   <si>
-    <t>Seized – Hospital</t>
-  </si>
-  <si>
-    <t>Seized – Signed over</t>
-  </si>
-  <si>
     <t>Seized – Eviction</t>
   </si>
   <si>
@@ -296,9 +356,6 @@
     <t>Seized - Hoarding</t>
   </si>
   <si>
-    <t>Return</t>
-  </si>
-  <si>
     <t>OTC - OS - SAFE</t>
   </si>
   <si>
@@ -312,9 +369,6 @@
   </si>
   <si>
     <t>Clinic - Case Assistance</t>
-  </si>
-  <si>
-    <t>Clinic - Case Assistance - Outreach</t>
   </si>
   <si>
     <t>Clinic - Outreach</t>
@@ -697,7 +751,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" customWidth="1"/>
@@ -717,7 +771,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -725,7 +779,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -741,7 +795,7 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>222</v>
+        <v>211</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -757,7 +811,7 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:2">
@@ -781,7 +835,7 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -797,7 +851,7 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -805,7 +859,7 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -821,18 +875,18 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
         <v>16</v>
       </c>
       <c r="B17">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -843,18 +897,18 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:3">
       <c r="A20" t="s">
         <v>20</v>
       </c>
       <c r="B20">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C20">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -865,51 +919,51 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:3">
       <c r="A22" t="s">
         <v>22</v>
       </c>
       <c r="B22">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="C22">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="A23" t="s">
         <v>23</v>
       </c>
       <c r="B23">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C23">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:3">
       <c r="A24" t="s">
         <v>24</v>
       </c>
       <c r="B24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C24">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
       <c r="A25" t="s">
         <v>25</v>
       </c>
       <c r="B25">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="C25">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
@@ -920,7 +974,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:3">
       <c r="A28" t="s">
         <v>29</v>
       </c>
@@ -931,7 +985,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:3">
       <c r="A29" t="s">
         <v>32</v>
       </c>
@@ -942,174 +996,230 @@
         <v>34</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C32" s="1" t="s">
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" t="s">
+        <v>36</v>
+      </c>
+      <c r="C30" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B31" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" t="s">
+        <v>41</v>
+      </c>
+      <c r="C32" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" t="s">
+        <v>41</v>
+      </c>
+      <c r="C33" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C36" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D36" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
-      <c r="A33" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
-        <v>73</v>
-      </c>
-      <c r="B34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>77</v>
-      </c>
-      <c r="C36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:4">
       <c r="A37" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="38" spans="1:3">
+      <c r="C37">
+        <v>1</v>
+      </c>
+      <c r="D37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="B39">
         <v>2</v>
       </c>
-      <c r="C39">
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
+      <c r="A41" t="s">
+        <v>100</v>
+      </c>
+      <c r="B41">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
+      <c r="A42" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
+      <c r="A43" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
+      <c r="A44" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
+      <c r="A45" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
+      <c r="A46" t="s">
+        <v>98</v>
+      </c>
+      <c r="D46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
+      <c r="A47" t="s">
+        <v>97</v>
+      </c>
+      <c r="C47">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
-      <c r="A40" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3">
-      <c r="A41" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3">
-      <c r="A42" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3">
-      <c r="A43" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3">
-      <c r="A44" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3">
-      <c r="A45" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3">
-      <c r="A46" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3">
-      <c r="A47" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:4">
       <c r="A48" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" t="s">
-        <v>70</v>
-      </c>
-      <c r="B50">
-        <v>11</v>
-      </c>
-      <c r="D50">
-        <v>9</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" t="s">
-        <v>76</v>
-      </c>
-      <c r="C51">
-        <v>1</v>
+        <v>111</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" t="s">
-        <v>94</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" t="s">
-        <v>95</v>
+        <v>79</v>
+      </c>
+      <c r="B53">
+        <v>3</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" t="s">
-        <v>96</v>
+        <v>81</v>
+      </c>
+      <c r="B54">
+        <v>5</v>
+      </c>
+      <c r="D54">
+        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" t="s">
-        <v>97</v>
+        <v>95</v>
+      </c>
+      <c r="B55">
+        <v>3</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" t="s">
-        <v>99</v>
+        <v>114</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" t="s">
-        <v>101</v>
+        <v>116</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" t="s">
+        <v>94</v>
+      </c>
+      <c r="B61">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="A63" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1119,547 +1229,567 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>50</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>83</v>
       </c>
       <c r="F2" t="s">
-        <v>76</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C3" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="E3" t="s">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="F3" t="s">
-        <v>77</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
       </c>
       <c r="C4" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="F4" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
       </c>
       <c r="C5" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="E5" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="F5" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
       <c r="C6" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="E6" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="F6" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="E7" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="E8" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>70</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
       <c r="C9" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="E9" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="C10" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B11" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="C11" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="F11" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="C12" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D12" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E12" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="C13" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="F13" t="s">
-        <v>70</v>
+        <v>97</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C14" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D14" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F14" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C15" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D15" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F15" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C16" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D16" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E16" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="C17" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E17" t="s">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="F17" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B18" t="s">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="C18" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D18" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E18" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="F18" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="B19" t="s">
         <v>20</v>
       </c>
       <c r="C19" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D19" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E19" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
       </c>
       <c r="C20" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E20" t="s">
-        <v>75</v>
+        <v>90</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B21" t="s">
         <v>20</v>
       </c>
       <c r="C21" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D21" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E21" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="F21" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
       </c>
       <c r="C22" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D22" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E22" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
       <c r="F22" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="C23" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D23" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E23" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="F23" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B24" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E24" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="F24" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="B25" t="s">
         <v>20</v>
       </c>
       <c r="C25" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D25" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E25" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B26" t="s">
         <v>20</v>
       </c>
       <c r="C26" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D26" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
       <c r="E26" t="s">
-        <v>75</v>
+        <v>92</v>
       </c>
       <c r="F26" t="s">
-        <v>70</v>
+        <v>81</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" t="s">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="C27" s="3">
-        <v>45847</v>
+        <v>45848</v>
       </c>
       <c r="D27" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="E27" t="s">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="F27" t="s">
-        <v>70</v>
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" t="s">
+        <v>40</v>
+      </c>
+      <c r="B28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28" s="3">
+        <v>45848</v>
+      </c>
+      <c r="D28" t="s">
+        <v>82</v>
+      </c>
+      <c r="E28" t="s">
+        <v>93</v>
+      </c>
+      <c r="F28" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>